<commit_message>
chore: regenerate data, remove 23 redundant player PNGs, fix Milos G
- Re-run parse-data to regenerate players/gameweeks/special-cards JSON
- Rename Minos G.png → Milos G.png (typo fix)
- Delete 23 player PNGs that have no matching player in the dataset

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/Vaksala KR-cupen 25_26.xlsx
+++ b/data/Vaksala KR-cupen 25_26.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1148" uniqueCount="112">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1147" uniqueCount="111">
   <si>
     <t>Knullrunkcupen 2025/2026</t>
   </si>
@@ -226,9 +226,6 @@
   </si>
   <si>
     <t>Georgios T</t>
-  </si>
-  <si>
-    <t>Benji L</t>
   </si>
   <si>
     <t>Jesper H</t>
@@ -19552,8 +19549,8 @@
 </f>
         <v>2</v>
       </c>
-      <c r="M225" s="57" t="s">
-        <v>70</v>
+      <c r="M225" s="53" t="s">
+        <v>53</v>
       </c>
       <c r="N225" s="10">
         <v>0.0</v>
@@ -19683,7 +19680,7 @@
         <v>Oavgjort</v>
       </c>
       <c r="H226" s="56" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="I226" s="9">
         <v>0.0</v>
@@ -19914,7 +19911,7 @@
         <v>Grön</v>
       </c>
       <c r="H228" s="38" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="I228" s="9">
         <v>1.0</v>
@@ -21390,7 +21387,7 @@
         <v>5.0</v>
       </c>
       <c r="R246" s="54" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="S246" s="11">
         <v>2.0</v>
@@ -21494,7 +21491,7 @@
         <v>3.0</v>
       </c>
       <c r="M247" s="53" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="N247" s="10">
         <v>2.0</v>
@@ -21604,7 +21601,7 @@
         <v>3.0</v>
       </c>
       <c r="M248" s="53" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="N248" s="10">
         <v>0.0</v>
@@ -23030,7 +23027,7 @@
         <v>Oavgjort</v>
       </c>
       <c r="H266" s="52" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="I266" s="9">
         <v>2.0</v>
@@ -23253,7 +23250,7 @@
         <v>Rosa</v>
       </c>
       <c r="H268" s="23" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="I268" s="9">
         <v>3.0</v>
@@ -24805,7 +24802,7 @@
         <v>7.0</v>
       </c>
       <c r="M287" s="57" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="N287" s="10">
         <v>3.0</v>
@@ -24820,7 +24817,7 @@
         <v>3.0</v>
       </c>
       <c r="R287" s="54" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="S287" s="11">
         <v>5.0</v>
@@ -24900,7 +24897,7 @@
         <v>Blå</v>
       </c>
       <c r="H288" s="38" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="I288" s="9">
         <v>0.0</v>
@@ -25009,7 +25006,7 @@
         <v>Blå</v>
       </c>
       <c r="H289" s="38" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="I289" s="9">
         <v>1.0</v>
@@ -26490,7 +26487,7 @@
         <v>6.0</v>
       </c>
       <c r="M307" s="53" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="N307" s="10">
         <v>1.0</v>
@@ -29923,7 +29920,7 @@
         <v>Grön</v>
       </c>
       <c r="H348" s="23" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="I348" s="9">
         <v>0.0</v>
@@ -29953,7 +29950,7 @@
         <v>2.0</v>
       </c>
       <c r="R348" s="54" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="S348" s="11">
         <v>5.0</v>
@@ -31400,7 +31397,7 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="58" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="B1" s="58" t="s">
         <v>3</v>
@@ -31415,7 +31412,7 @@
         <v>16</v>
       </c>
       <c r="F1" s="58" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="G1" s="58" t="s">
         <v>17</v>
@@ -31424,13 +31421,13 @@
         <v>10</v>
       </c>
       <c r="J1" s="59" t="s">
+        <v>79</v>
+      </c>
+      <c r="K1" s="59" t="s">
         <v>80</v>
       </c>
-      <c r="K1" s="59" t="s">
-        <v>81</v>
-      </c>
       <c r="L1" s="58" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="M1" s="58" t="s">
         <v>3</v>
@@ -31445,7 +31442,7 @@
         <v>16</v>
       </c>
       <c r="Q1" s="58" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="R1" s="58" t="s">
         <v>17</v>
@@ -31502,7 +31499,7 @@
         <v>94</v>
       </c>
       <c r="L2" s="60" t="str">
-        <f t="array" ref="L2:L55">SORT(UNIQUE(Spelarstatistik!A2:A179))</f>
+        <f t="array" ref="L2:L54">SORT(UNIQUE(Spelarstatistik!A2:A179))</f>
         <v>Achillie X</v>
       </c>
       <c r="M2" s="60">
@@ -31846,22 +31843,22 @@
       <c r="N6" s="60">
         <f>SUMIF(Spelarstatistik!A$2:A179, L6, Spelarstatistik!C$2:C179)
 </f>
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="O6" s="60">
         <f>SUMIF(Spelarstatistik!A$2:A179, L6, Spelarstatistik!D$2:D179)
 </f>
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="P6" s="60">
         <f>SUMIF(Spelarstatistik!A$2:A179, L6, Spelarstatistik!E$2:E179)
 </f>
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="Q6" s="60">
         <f>COUNTIF(Spelarstatistik!A$2:A179, L6)
 </f>
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="R6" s="60">
         <f>SUMIF(Matcher!AC$5:AC179, L6, Matcher!AH$5:AH179)
@@ -31870,7 +31867,7 @@
       </c>
       <c r="S6" s="60">
         <f t="shared" si="4"/>
-        <v>36</v>
+        <v>43</v>
       </c>
     </row>
     <row r="7">
@@ -31919,41 +31916,41 @@
         <v>84</v>
       </c>
       <c r="L7" s="60" t="s">
-        <v>70</v>
+        <v>27</v>
       </c>
       <c r="M7" s="60">
         <f>SUMIF(Spelarstatistik!A$2:A179, L7, Spelarstatistik!B$2:B179)
 </f>
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="N7" s="60">
         <f>SUMIF(Spelarstatistik!A$2:A179, L7, Spelarstatistik!C$2:C179)
 </f>
-        <v>2</v>
+        <v>9</v>
       </c>
       <c r="O7" s="60">
         <f>SUMIF(Spelarstatistik!A$2:A179, L7, Spelarstatistik!D$2:D179)
 </f>
-        <v>1</v>
+        <v>22</v>
       </c>
       <c r="P7" s="60">
         <f>SUMIF(Spelarstatistik!A$2:A179, L7, Spelarstatistik!E$2:E179)
 </f>
-        <v>3</v>
+        <v>14</v>
       </c>
       <c r="Q7" s="60">
         <f>COUNTIF(Spelarstatistik!A$2:A179, L7)
 </f>
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="R7" s="60">
         <f>SUMIF(Matcher!AC$5:AC179, L7, Matcher!AH$5:AH179)
 </f>
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="S7" s="60">
         <f t="shared" si="4"/>
-        <v>8</v>
+        <v>57</v>
       </c>
     </row>
     <row r="8">
@@ -32002,41 +31999,41 @@
         <v>65</v>
       </c>
       <c r="L8" s="60" t="s">
-        <v>27</v>
+        <v>45</v>
       </c>
       <c r="M8" s="60">
         <f>SUMIF(Spelarstatistik!A$2:A179, L8, Spelarstatistik!B$2:B179)
 </f>
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="N8" s="60">
         <f>SUMIF(Spelarstatistik!A$2:A179, L8, Spelarstatistik!C$2:C179)
 </f>
-        <v>9</v>
+        <v>1</v>
       </c>
       <c r="O8" s="60">
         <f>SUMIF(Spelarstatistik!A$2:A179, L8, Spelarstatistik!D$2:D179)
 </f>
-        <v>22</v>
+        <v>13</v>
       </c>
       <c r="P8" s="60">
         <f>SUMIF(Spelarstatistik!A$2:A179, L8, Spelarstatistik!E$2:E179)
 </f>
-        <v>14</v>
+        <v>26</v>
       </c>
       <c r="Q8" s="60">
         <f>COUNTIF(Spelarstatistik!A$2:A179, L8)
 </f>
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="R8" s="60">
         <f>SUMIF(Matcher!AC$5:AC179, L8, Matcher!AH$5:AH179)
 </f>
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="S8" s="60">
         <f t="shared" si="4"/>
-        <v>57</v>
+        <v>46</v>
       </c>
     </row>
     <row r="9">
@@ -32085,32 +32082,32 @@
         <v>79</v>
       </c>
       <c r="L9" s="60" t="s">
-        <v>45</v>
+        <v>25</v>
       </c>
       <c r="M9" s="60">
         <f>SUMIF(Spelarstatistik!A$2:A179, L9, Spelarstatistik!B$2:B179)
 </f>
-        <v>8</v>
+        <v>24</v>
       </c>
       <c r="N9" s="60">
         <f>SUMIF(Spelarstatistik!A$2:A179, L9, Spelarstatistik!C$2:C179)
 </f>
-        <v>1</v>
+        <v>20</v>
       </c>
       <c r="O9" s="60">
         <f>SUMIF(Spelarstatistik!A$2:A179, L9, Spelarstatistik!D$2:D179)
 </f>
-        <v>13</v>
+        <v>37</v>
       </c>
       <c r="P9" s="60">
         <f>SUMIF(Spelarstatistik!A$2:A179, L9, Spelarstatistik!E$2:E179)
 </f>
-        <v>26</v>
+        <v>36</v>
       </c>
       <c r="Q9" s="60">
         <f>COUNTIF(Spelarstatistik!A$2:A179, L9)
 </f>
-        <v>6</v>
+        <v>14</v>
       </c>
       <c r="R9" s="60">
         <f>SUMIF(Matcher!AC$5:AC179, L9, Matcher!AH$5:AH179)
@@ -32119,7 +32116,7 @@
       </c>
       <c r="S9" s="60">
         <f t="shared" si="4"/>
-        <v>46</v>
+        <v>133</v>
       </c>
     </row>
     <row r="10">
@@ -32168,32 +32165,32 @@
         <v>80</v>
       </c>
       <c r="L10" s="60" t="s">
-        <v>25</v>
+        <v>57</v>
       </c>
       <c r="M10" s="60">
         <f>SUMIF(Spelarstatistik!A$2:A179, L10, Spelarstatistik!B$2:B179)
 </f>
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="N10" s="60">
         <f>SUMIF(Spelarstatistik!A$2:A179, L10, Spelarstatistik!C$2:C179)
 </f>
-        <v>20</v>
+        <v>12</v>
       </c>
       <c r="O10" s="60">
         <f>SUMIF(Spelarstatistik!A$2:A179, L10, Spelarstatistik!D$2:D179)
 </f>
-        <v>37</v>
+        <v>19</v>
       </c>
       <c r="P10" s="60">
         <f>SUMIF(Spelarstatistik!A$2:A179, L10, Spelarstatistik!E$2:E179)
 </f>
-        <v>36</v>
+        <v>15</v>
       </c>
       <c r="Q10" s="60">
         <f>COUNTIF(Spelarstatistik!A$2:A179, L10)
 </f>
-        <v>14</v>
+        <v>6</v>
       </c>
       <c r="R10" s="60">
         <f>SUMIF(Matcher!AC$5:AC179, L10, Matcher!AH$5:AH179)
@@ -32202,7 +32199,7 @@
       </c>
       <c r="S10" s="60">
         <f t="shared" si="4"/>
-        <v>133</v>
+        <v>78</v>
       </c>
     </row>
     <row r="11">
@@ -32251,41 +32248,41 @@
         <v>60</v>
       </c>
       <c r="L11" s="60" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="M11" s="60">
         <f>SUMIF(Spelarstatistik!A$2:A179, L11, Spelarstatistik!B$2:B179)
 </f>
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="N11" s="60">
         <f>SUMIF(Spelarstatistik!A$2:A179, L11, Spelarstatistik!C$2:C179)
 </f>
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="O11" s="60">
         <f>SUMIF(Spelarstatistik!A$2:A179, L11, Spelarstatistik!D$2:D179)
 </f>
-        <v>19</v>
+        <v>30</v>
       </c>
       <c r="P11" s="60">
         <f>SUMIF(Spelarstatistik!A$2:A179, L11, Spelarstatistik!E$2:E179)
 </f>
-        <v>15</v>
+        <v>20</v>
       </c>
       <c r="Q11" s="60">
         <f>COUNTIF(Spelarstatistik!A$2:A179, L11)
 </f>
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="R11" s="60">
         <f>SUMIF(Matcher!AC$5:AC179, L11, Matcher!AH$5:AH179)
 </f>
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="S11" s="60">
         <f t="shared" si="4"/>
-        <v>78</v>
+        <v>97</v>
       </c>
     </row>
     <row r="12">
@@ -32334,41 +32331,41 @@
         <v>67</v>
       </c>
       <c r="L12" s="60" t="s">
-        <v>55</v>
+        <v>38</v>
       </c>
       <c r="M12" s="60">
         <f>SUMIF(Spelarstatistik!A$2:A179, L12, Spelarstatistik!B$2:B179)
 </f>
-        <v>23</v>
+        <v>0</v>
       </c>
       <c r="N12" s="60">
         <f>SUMIF(Spelarstatistik!A$2:A179, L12, Spelarstatistik!C$2:C179)
 </f>
-        <v>11</v>
+        <v>0</v>
       </c>
       <c r="O12" s="60">
         <f>SUMIF(Spelarstatistik!A$2:A179, L12, Spelarstatistik!D$2:D179)
 </f>
-        <v>30</v>
+        <v>6</v>
       </c>
       <c r="P12" s="60">
         <f>SUMIF(Spelarstatistik!A$2:A179, L12, Spelarstatistik!E$2:E179)
 </f>
-        <v>20</v>
+        <v>9</v>
       </c>
       <c r="Q12" s="60">
         <f>COUNTIF(Spelarstatistik!A$2:A179, L12)
 </f>
-        <v>9</v>
+        <v>2</v>
       </c>
       <c r="R12" s="60">
         <f>SUMIF(Matcher!AC$5:AC179, L12, Matcher!AH$5:AH179)
 </f>
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="S12" s="60">
         <f t="shared" si="4"/>
-        <v>97</v>
+        <v>18</v>
       </c>
     </row>
     <row r="13">
@@ -32417,41 +32414,41 @@
         <v>84</v>
       </c>
       <c r="L13" s="60" t="s">
-        <v>38</v>
+        <v>60</v>
       </c>
       <c r="M13" s="60">
         <f>SUMIF(Spelarstatistik!A$2:A179, L13, Spelarstatistik!B$2:B179)
 </f>
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="N13" s="60">
         <f>SUMIF(Spelarstatistik!A$2:A179, L13, Spelarstatistik!C$2:C179)
 </f>
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="O13" s="60">
         <f>SUMIF(Spelarstatistik!A$2:A179, L13, Spelarstatistik!D$2:D179)
 </f>
-        <v>6</v>
+        <v>14</v>
       </c>
       <c r="P13" s="60">
         <f>SUMIF(Spelarstatistik!A$2:A179, L13, Spelarstatistik!E$2:E179)
 </f>
-        <v>9</v>
+        <v>17</v>
       </c>
       <c r="Q13" s="60">
         <f>COUNTIF(Spelarstatistik!A$2:A179, L13)
 </f>
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="R13" s="60">
         <f>SUMIF(Matcher!AC$5:AC179, L13, Matcher!AH$5:AH179)
 </f>
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="S13" s="60">
         <f t="shared" si="4"/>
-        <v>18</v>
+        <v>41</v>
       </c>
     </row>
     <row r="14">
@@ -32500,7 +32497,7 @@
         <v>59</v>
       </c>
       <c r="L14" s="60" t="s">
-        <v>60</v>
+        <v>30</v>
       </c>
       <c r="M14" s="60">
         <f>SUMIF(Spelarstatistik!A$2:A179, L14, Spelarstatistik!B$2:B179)
@@ -32510,31 +32507,31 @@
       <c r="N14" s="60">
         <f>SUMIF(Spelarstatistik!A$2:A179, L14, Spelarstatistik!C$2:C179)
 </f>
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="O14" s="60">
         <f>SUMIF(Spelarstatistik!A$2:A179, L14, Spelarstatistik!D$2:D179)
 </f>
-        <v>14</v>
+        <v>56</v>
       </c>
       <c r="P14" s="60">
         <f>SUMIF(Spelarstatistik!A$2:A179, L14, Spelarstatistik!E$2:E179)
 </f>
-        <v>17</v>
+        <v>57</v>
       </c>
       <c r="Q14" s="60">
         <f>COUNTIF(Spelarstatistik!A$2:A179, L14)
 </f>
-        <v>5</v>
+        <v>14</v>
       </c>
       <c r="R14" s="60">
         <f>SUMIF(Matcher!AC$5:AC179, L14, Matcher!AH$5:AH179)
 </f>
-        <v>0</v>
+        <v>72</v>
       </c>
       <c r="S14" s="60">
         <f t="shared" si="4"/>
-        <v>41</v>
+        <v>146</v>
       </c>
     </row>
     <row r="15">
@@ -32583,41 +32580,41 @@
         <v>70</v>
       </c>
       <c r="L15" s="60" t="s">
-        <v>30</v>
+        <v>39</v>
       </c>
       <c r="M15" s="60">
         <f>SUMIF(Spelarstatistik!A$2:A179, L15, Spelarstatistik!B$2:B179)
 </f>
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="N15" s="60">
         <f>SUMIF(Spelarstatistik!A$2:A179, L15, Spelarstatistik!C$2:C179)
 </f>
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="O15" s="60">
         <f>SUMIF(Spelarstatistik!A$2:A179, L15, Spelarstatistik!D$2:D179)
 </f>
-        <v>56</v>
+        <v>8</v>
       </c>
       <c r="P15" s="60">
         <f>SUMIF(Spelarstatistik!A$2:A179, L15, Spelarstatistik!E$2:E179)
 </f>
-        <v>57</v>
+        <v>6</v>
       </c>
       <c r="Q15" s="60">
         <f>COUNTIF(Spelarstatistik!A$2:A179, L15)
 </f>
-        <v>14</v>
+        <v>2</v>
       </c>
       <c r="R15" s="60">
         <f>SUMIF(Matcher!AC$5:AC179, L15, Matcher!AH$5:AH179)
 </f>
-        <v>72</v>
+        <v>0</v>
       </c>
       <c r="S15" s="60">
         <f t="shared" si="4"/>
-        <v>146</v>
+        <v>26</v>
       </c>
     </row>
     <row r="16">
@@ -32666,32 +32663,32 @@
         <v>65</v>
       </c>
       <c r="L16" s="60" t="s">
-        <v>39</v>
+        <v>49</v>
       </c>
       <c r="M16" s="60">
         <f>SUMIF(Spelarstatistik!A$2:A179, L16, Spelarstatistik!B$2:B179)
 </f>
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="N16" s="60">
         <f>SUMIF(Spelarstatistik!A$2:A179, L16, Spelarstatistik!C$2:C179)
 </f>
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="O16" s="60">
         <f>SUMIF(Spelarstatistik!A$2:A179, L16, Spelarstatistik!D$2:D179)
 </f>
-        <v>8</v>
+        <v>16</v>
       </c>
       <c r="P16" s="60">
         <f>SUMIF(Spelarstatistik!A$2:A179, L16, Spelarstatistik!E$2:E179)
 </f>
-        <v>6</v>
+        <v>11</v>
       </c>
       <c r="Q16" s="60">
         <f>COUNTIF(Spelarstatistik!A$2:A179, L16)
 </f>
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="R16" s="60">
         <f>SUMIF(Matcher!AC$5:AC179, L16, Matcher!AH$5:AH179)
@@ -32700,7 +32697,7 @@
       </c>
       <c r="S16" s="60">
         <f t="shared" si="4"/>
-        <v>26</v>
+        <v>46</v>
       </c>
     </row>
     <row r="17">
@@ -32749,32 +32746,32 @@
         <v>64</v>
       </c>
       <c r="L17" s="60" t="s">
-        <v>49</v>
+        <v>46</v>
       </c>
       <c r="M17" s="60">
         <f>SUMIF(Spelarstatistik!A$2:A179, L17, Spelarstatistik!B$2:B179)
 </f>
-        <v>11</v>
+        <v>3</v>
       </c>
       <c r="N17" s="60">
         <f>SUMIF(Spelarstatistik!A$2:A179, L17, Spelarstatistik!C$2:C179)
 </f>
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="O17" s="60">
         <f>SUMIF(Spelarstatistik!A$2:A179, L17, Spelarstatistik!D$2:D179)
 </f>
-        <v>16</v>
+        <v>6</v>
       </c>
       <c r="P17" s="60">
         <f>SUMIF(Spelarstatistik!A$2:A179, L17, Spelarstatistik!E$2:E179)
 </f>
-        <v>11</v>
+        <v>0</v>
       </c>
       <c r="Q17" s="60">
         <f>COUNTIF(Spelarstatistik!A$2:A179, L17)
 </f>
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="R17" s="60">
         <f>SUMIF(Matcher!AC$5:AC179, L17, Matcher!AH$5:AH179)
@@ -32783,7 +32780,7 @@
       </c>
       <c r="S17" s="60">
         <f t="shared" si="4"/>
-        <v>46</v>
+        <v>15</v>
       </c>
     </row>
     <row r="18">
@@ -32832,32 +32829,32 @@
         <v>80</v>
       </c>
       <c r="L18" s="60" t="s">
-        <v>46</v>
+        <v>65</v>
       </c>
       <c r="M18" s="60">
         <f>SUMIF(Spelarstatistik!A$2:A179, L18, Spelarstatistik!B$2:B179)
 </f>
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="N18" s="60">
         <f>SUMIF(Spelarstatistik!A$2:A179, L18, Spelarstatistik!C$2:C179)
 </f>
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="O18" s="60">
         <f>SUMIF(Spelarstatistik!A$2:A179, L18, Spelarstatistik!D$2:D179)
 </f>
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="P18" s="60">
         <f>SUMIF(Spelarstatistik!A$2:A179, L18, Spelarstatistik!E$2:E179)
 </f>
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="Q18" s="60">
         <f>COUNTIF(Spelarstatistik!A$2:A179, L18)
 </f>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="R18" s="60">
         <f>SUMIF(Matcher!AC$5:AC179, L18, Matcher!AH$5:AH179)
@@ -32866,7 +32863,7 @@
       </c>
       <c r="S18" s="60">
         <f t="shared" si="4"/>
-        <v>15</v>
+        <v>17</v>
       </c>
     </row>
     <row r="19">
@@ -32915,32 +32912,32 @@
         <v>67</v>
       </c>
       <c r="L19" s="60" t="s">
-        <v>65</v>
+        <v>59</v>
       </c>
       <c r="M19" s="60">
         <f>SUMIF(Spelarstatistik!A$2:A179, L19, Spelarstatistik!B$2:B179)
 </f>
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="N19" s="60">
         <f>SUMIF(Spelarstatistik!A$2:A179, L19, Spelarstatistik!C$2:C179)
 </f>
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="O19" s="60">
         <f>SUMIF(Spelarstatistik!A$2:A179, L19, Spelarstatistik!D$2:D179)
 </f>
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="P19" s="60">
         <f>SUMIF(Spelarstatistik!A$2:A179, L19, Spelarstatistik!E$2:E179)
 </f>
-        <v>6</v>
+        <v>14</v>
       </c>
       <c r="Q19" s="60">
         <f>COUNTIF(Spelarstatistik!A$2:A179, L19)
 </f>
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="R19" s="60">
         <f>SUMIF(Matcher!AC$5:AC179, L19, Matcher!AH$5:AH179)
@@ -32949,7 +32946,7 @@
       </c>
       <c r="S19" s="60">
         <f t="shared" si="4"/>
-        <v>17</v>
+        <v>37</v>
       </c>
     </row>
     <row r="20">
@@ -32998,32 +32995,32 @@
         <v>55</v>
       </c>
       <c r="L20" s="60" t="s">
-        <v>59</v>
+        <v>69</v>
       </c>
       <c r="M20" s="60">
         <f>SUMIF(Spelarstatistik!A$2:A179, L20, Spelarstatistik!B$2:B179)
 </f>
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="N20" s="60">
         <f>SUMIF(Spelarstatistik!A$2:A179, L20, Spelarstatistik!C$2:C179)
 </f>
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="O20" s="60">
         <f>SUMIF(Spelarstatistik!A$2:A179, L20, Spelarstatistik!D$2:D179)
 </f>
-        <v>12</v>
+        <v>5</v>
       </c>
       <c r="P20" s="60">
         <f>SUMIF(Spelarstatistik!A$2:A179, L20, Spelarstatistik!E$2:E179)
 </f>
-        <v>14</v>
+        <v>1</v>
       </c>
       <c r="Q20" s="60">
         <f>COUNTIF(Spelarstatistik!A$2:A179, L20)
 </f>
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="R20" s="60">
         <f>SUMIF(Matcher!AC$5:AC179, L20, Matcher!AH$5:AH179)
@@ -33032,7 +33029,7 @@
       </c>
       <c r="S20" s="60">
         <f t="shared" si="4"/>
-        <v>37</v>
+        <v>10</v>
       </c>
     </row>
     <row r="21">
@@ -33081,27 +33078,27 @@
         <v>65</v>
       </c>
       <c r="L21" s="63" t="s">
-        <v>69</v>
+        <v>76</v>
       </c>
       <c r="M21" s="60">
         <f>SUMIF(Spelarstatistik!A$2:A179, L21, Spelarstatistik!B$2:B179)
 </f>
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="N21" s="60">
         <f>SUMIF(Spelarstatistik!A$2:A179, L21, Spelarstatistik!C$2:C179)
 </f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="O21" s="60">
         <f>SUMIF(Spelarstatistik!A$2:A179, L21, Spelarstatistik!D$2:D179)
 </f>
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="P21" s="60">
         <f>SUMIF(Spelarstatistik!A$2:A179, L21, Spelarstatistik!E$2:E179)
 </f>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="Q21" s="60">
         <f>COUNTIF(Spelarstatistik!A$2:A179, L21)
@@ -33115,7 +33112,7 @@
       </c>
       <c r="S21" s="60">
         <f t="shared" si="4"/>
-        <v>10</v>
+        <v>12</v>
       </c>
     </row>
     <row r="22">
@@ -33164,12 +33161,12 @@
         <v>80</v>
       </c>
       <c r="L22" s="63" t="s">
-        <v>77</v>
+        <v>68</v>
       </c>
       <c r="M22" s="60">
         <f>SUMIF(Spelarstatistik!A$2:A179, L22, Spelarstatistik!B$2:B179)
 </f>
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="N22" s="60">
         <f>SUMIF(Spelarstatistik!A$2:A179, L22, Spelarstatistik!C$2:C179)
@@ -33179,12 +33176,12 @@
       <c r="O22" s="60">
         <f>SUMIF(Spelarstatistik!A$2:A179, L22, Spelarstatistik!D$2:D179)
 </f>
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="P22" s="60">
         <f>SUMIF(Spelarstatistik!A$2:A179, L22, Spelarstatistik!E$2:E179)
 </f>
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="Q22" s="60">
         <f>COUNTIF(Spelarstatistik!A$2:A179, L22)
@@ -33198,29 +33195,29 @@
       </c>
       <c r="S22" s="60">
         <f t="shared" si="4"/>
-        <v>12</v>
+        <v>7</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="60" t="str">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"Albert A")</f>
-        <v>Albert A</v>
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"Benjamin L")</f>
+        <v>Benjamin L</v>
       </c>
       <c r="B23" s="61">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),3.0)</f>
-        <v>3</v>
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),1.0)</f>
+        <v>1</v>
       </c>
       <c r="C23" s="61">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),2.0)</f>
-        <v>2</v>
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),4.0)</f>
+        <v>4</v>
       </c>
       <c r="D23" s="61">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),13.0)</f>
-        <v>13</v>
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),16.0)</f>
+        <v>16</v>
       </c>
       <c r="E23" s="61">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),19.0)</f>
-        <v>19</v>
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),14.0)</f>
+        <v>14</v>
       </c>
       <c r="F23" s="61">
         <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),6.0)</f>
@@ -33231,8 +33228,8 @@
         <v>0</v>
       </c>
       <c r="H23" s="61">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),42.0)</f>
-        <v>42</v>
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),43.0)</f>
+        <v>43</v>
       </c>
       <c r="I23" s="60" t="str">
         <f t="shared" si="1"/>
@@ -33240,39 +33237,39 @@
       </c>
       <c r="J23" s="62">
         <f t="shared" si="2"/>
-        <v>7</v>
+        <v>7.2</v>
       </c>
       <c r="K23" s="62">
         <f t="shared" si="3"/>
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="L23" s="60" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="M23" s="60">
         <f>SUMIF(Spelarstatistik!A$2:A179, L23, Spelarstatistik!B$2:B179)
 </f>
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="N23" s="60">
         <f>SUMIF(Spelarstatistik!A$2:A179, L23, Spelarstatistik!C$2:C179)
 </f>
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="O23" s="60">
         <f>SUMIF(Spelarstatistik!A$2:A179, L23, Spelarstatistik!D$2:D179)
 </f>
-        <v>3</v>
+        <v>19</v>
       </c>
       <c r="P23" s="60">
         <f>SUMIF(Spelarstatistik!A$2:A179, L23, Spelarstatistik!E$2:E179)
 </f>
-        <v>1</v>
+        <v>14</v>
       </c>
       <c r="Q23" s="60">
         <f>COUNTIF(Spelarstatistik!A$2:A179, L23)
 </f>
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="R23" s="60">
         <f>SUMIF(Matcher!AC$5:AC179, L23, Matcher!AH$5:AH179)
@@ -33281,33 +33278,33 @@
       </c>
       <c r="S23" s="60">
         <f t="shared" si="4"/>
-        <v>7</v>
+        <v>48</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="60" t="str">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"Pontus B")</f>
-        <v>Pontus B</v>
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"Albert A")</f>
+        <v>Albert A</v>
       </c>
       <c r="B24" s="61">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),9.0)</f>
-        <v>9</v>
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),3.0)</f>
+        <v>3</v>
       </c>
       <c r="C24" s="61">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),8.0)</f>
-        <v>8</v>
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),2.0)</f>
+        <v>2</v>
       </c>
       <c r="D24" s="61">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),9.0)</f>
-        <v>9</v>
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),13.0)</f>
+        <v>13</v>
       </c>
       <c r="E24" s="61">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),12.0)</f>
-        <v>12</v>
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),19.0)</f>
+        <v>19</v>
       </c>
       <c r="F24" s="61">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),4.0)</f>
-        <v>4</v>
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),6.0)</f>
+        <v>6</v>
       </c>
       <c r="G24" s="61">
         <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0)</f>
@@ -33323,39 +33320,39 @@
       </c>
       <c r="J24" s="62">
         <f t="shared" si="2"/>
-        <v>10.5</v>
+        <v>7</v>
       </c>
       <c r="K24" s="62">
         <f t="shared" si="3"/>
-        <v>73</v>
+        <v>50</v>
       </c>
       <c r="L24" s="60" t="s">
-        <v>66</v>
+        <v>47</v>
       </c>
       <c r="M24" s="60">
         <f>SUMIF(Spelarstatistik!A$2:A179, L24, Spelarstatistik!B$2:B179)
 </f>
-        <v>9</v>
+        <v>1</v>
       </c>
       <c r="N24" s="60">
         <f>SUMIF(Spelarstatistik!A$2:A179, L24, Spelarstatistik!C$2:C179)
 </f>
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="O24" s="60">
         <f>SUMIF(Spelarstatistik!A$2:A179, L24, Spelarstatistik!D$2:D179)
 </f>
-        <v>19</v>
+        <v>0</v>
       </c>
       <c r="P24" s="60">
         <f>SUMIF(Spelarstatistik!A$2:A179, L24, Spelarstatistik!E$2:E179)
 </f>
-        <v>14</v>
+        <v>7</v>
       </c>
       <c r="Q24" s="60">
         <f>COUNTIF(Spelarstatistik!A$2:A179, L24)
 </f>
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="R24" s="60">
         <f>SUMIF(Matcher!AC$5:AC179, L24, Matcher!AH$5:AH179)
@@ -33364,29 +33361,29 @@
       </c>
       <c r="S24" s="60">
         <f t="shared" si="4"/>
-        <v>48</v>
+        <v>7</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="60" t="str">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"Shoresh A")</f>
-        <v>Shoresh A</v>
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"Pontus B")</f>
+        <v>Pontus B</v>
       </c>
       <c r="B25" s="61">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),6.0)</f>
-        <v>6</v>
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),9.0)</f>
+        <v>9</v>
       </c>
       <c r="C25" s="61">
         <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),8.0)</f>
         <v>8</v>
       </c>
       <c r="D25" s="61">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),15.0)</f>
-        <v>15</v>
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),9.0)</f>
+        <v>9</v>
       </c>
       <c r="E25" s="61">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),8.0)</f>
-        <v>8</v>
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),12.0)</f>
+        <v>12</v>
       </c>
       <c r="F25" s="61">
         <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),4.0)</f>
@@ -33413,32 +33410,32 @@
         <v>73</v>
       </c>
       <c r="L25" s="60" t="s">
-        <v>47</v>
+        <v>41</v>
       </c>
       <c r="M25" s="60">
         <f>SUMIF(Spelarstatistik!A$2:A179, L25, Spelarstatistik!B$2:B179)
 </f>
-        <v>1</v>
+        <v>13</v>
       </c>
       <c r="N25" s="60">
         <f>SUMIF(Spelarstatistik!A$2:A179, L25, Spelarstatistik!C$2:C179)
 </f>
-        <v>1</v>
+        <v>11</v>
       </c>
       <c r="O25" s="60">
         <f>SUMIF(Spelarstatistik!A$2:A179, L25, Spelarstatistik!D$2:D179)
 </f>
-        <v>0</v>
+        <v>17</v>
       </c>
       <c r="P25" s="60">
         <f>SUMIF(Spelarstatistik!A$2:A179, L25, Spelarstatistik!E$2:E179)
 </f>
-        <v>7</v>
+        <v>27</v>
       </c>
       <c r="Q25" s="60">
         <f>COUNTIF(Spelarstatistik!A$2:A179, L25)
 </f>
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="R25" s="60">
         <f>SUMIF(Matcher!AC$5:AC179, L25, Matcher!AH$5:AH179)
@@ -33447,41 +33444,41 @@
       </c>
       <c r="S25" s="60">
         <f t="shared" si="4"/>
-        <v>7</v>
+        <v>68</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="60" t="str">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"Emil A")</f>
-        <v>Emil A</v>
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"Shoresh A")</f>
+        <v>Shoresh A</v>
       </c>
       <c r="B26" s="64">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),3.0)</f>
-        <v>3</v>
-      </c>
-      <c r="C26" s="61">
         <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),6.0)</f>
         <v>6</v>
       </c>
+      <c r="C26" s="61">
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),8.0)</f>
+        <v>8</v>
+      </c>
       <c r="D26" s="61">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),14.0)</f>
-        <v>14</v>
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),15.0)</f>
+        <v>15</v>
       </c>
       <c r="E26" s="61">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),17.0)</f>
-        <v>17</v>
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),8.0)</f>
+        <v>8</v>
       </c>
       <c r="F26" s="61">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),5.0)</f>
-        <v>5</v>
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),4.0)</f>
+        <v>4</v>
       </c>
       <c r="G26" s="61">
         <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0)</f>
         <v>0</v>
       </c>
       <c r="H26" s="61">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),41.0)</f>
-        <v>41</v>
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),42.0)</f>
+        <v>42</v>
       </c>
       <c r="I26" s="60" t="str">
         <f t="shared" si="1"/>
@@ -33489,39 +33486,39 @@
       </c>
       <c r="J26" s="62">
         <f t="shared" si="2"/>
-        <v>8.2</v>
+        <v>10.5</v>
       </c>
       <c r="K26" s="62">
         <f t="shared" si="3"/>
+        <v>73</v>
+      </c>
+      <c r="L26" s="60" t="s">
         <v>58</v>
-      </c>
-      <c r="L26" s="60" t="s">
-        <v>41</v>
       </c>
       <c r="M26" s="60">
         <f>SUMIF(Spelarstatistik!A$2:A179, L26, Spelarstatistik!B$2:B179)
 </f>
-        <v>13</v>
+        <v>27</v>
       </c>
       <c r="N26" s="60">
         <f>SUMIF(Spelarstatistik!A$2:A179, L26, Spelarstatistik!C$2:C179)
 </f>
-        <v>11</v>
+        <v>24</v>
       </c>
       <c r="O26" s="60">
         <f>SUMIF(Spelarstatistik!A$2:A179, L26, Spelarstatistik!D$2:D179)
 </f>
-        <v>17</v>
+        <v>35</v>
       </c>
       <c r="P26" s="60">
         <f>SUMIF(Spelarstatistik!A$2:A179, L26, Spelarstatistik!E$2:E179)
 </f>
-        <v>27</v>
+        <v>39</v>
       </c>
       <c r="Q26" s="60">
         <f>COUNTIF(Spelarstatistik!A$2:A179, L26)
 </f>
-        <v>7</v>
+        <v>12</v>
       </c>
       <c r="R26" s="60">
         <f>SUMIF(Matcher!AC$5:AC179, L26, Matcher!AH$5:AH179)
@@ -33530,41 +33527,41 @@
       </c>
       <c r="S26" s="60">
         <f t="shared" si="4"/>
-        <v>68</v>
+        <v>129</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="60" t="str">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"Joel C")</f>
-        <v>Joel C</v>
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"Emil A")</f>
+        <v>Emil A</v>
       </c>
       <c r="B27" s="64">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),4.0)</f>
-        <v>4</v>
-      </c>
-      <c r="C27" s="61">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),13.0)</f>
-        <v>13</v>
-      </c>
-      <c r="D27" s="61">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),12.0)</f>
-        <v>12</v>
-      </c>
-      <c r="E27" s="61">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),7.0)</f>
-        <v>7</v>
-      </c>
-      <c r="F27" s="61">
         <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),3.0)</f>
         <v>3</v>
       </c>
+      <c r="C27" s="61">
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),6.0)</f>
+        <v>6</v>
+      </c>
+      <c r="D27" s="61">
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),14.0)</f>
+        <v>14</v>
+      </c>
+      <c r="E27" s="61">
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),17.0)</f>
+        <v>17</v>
+      </c>
+      <c r="F27" s="61">
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),5.0)</f>
+        <v>5</v>
+      </c>
       <c r="G27" s="61">
         <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0)</f>
         <v>0</v>
       </c>
       <c r="H27" s="61">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),38.0)</f>
-        <v>38</v>
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),41.0)</f>
+        <v>41</v>
       </c>
       <c r="I27" s="60" t="str">
         <f t="shared" si="1"/>
@@ -33572,39 +33569,39 @@
       </c>
       <c r="J27" s="62">
         <f t="shared" si="2"/>
-        <v>12.7</v>
+        <v>8.2</v>
       </c>
       <c r="K27" s="62">
         <f t="shared" si="3"/>
-        <v>79</v>
+        <v>58</v>
       </c>
       <c r="L27" s="60" t="s">
-        <v>58</v>
+        <v>36</v>
       </c>
       <c r="M27" s="60">
         <f>SUMIF(Spelarstatistik!A$2:A179, L27, Spelarstatistik!B$2:B179)
 </f>
-        <v>27</v>
+        <v>36</v>
       </c>
       <c r="N27" s="60">
         <f>SUMIF(Spelarstatistik!A$2:A179, L27, Spelarstatistik!C$2:C179)
 </f>
-        <v>24</v>
+        <v>37</v>
       </c>
       <c r="O27" s="60">
         <f>SUMIF(Spelarstatistik!A$2:A179, L27, Spelarstatistik!D$2:D179)
 </f>
-        <v>35</v>
+        <v>52</v>
       </c>
       <c r="P27" s="60">
         <f>SUMIF(Spelarstatistik!A$2:A179, L27, Spelarstatistik!E$2:E179)
 </f>
-        <v>39</v>
+        <v>32</v>
       </c>
       <c r="Q27" s="60">
         <f>COUNTIF(Spelarstatistik!A$2:A179, L27)
 </f>
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="R27" s="60">
         <f>SUMIF(Matcher!AC$5:AC179, L27, Matcher!AH$5:AH179)
@@ -33613,120 +33610,120 @@
       </c>
       <c r="S27" s="60">
         <f t="shared" si="4"/>
-        <v>129</v>
+        <v>174</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="60" t="str">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"George T")</f>
-        <v>George T</v>
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"Joel C")</f>
+        <v>Joel C</v>
       </c>
       <c r="B28" s="64">
         <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),4.0)</f>
         <v>4</v>
       </c>
       <c r="C28" s="61">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),7.0)</f>
-        <v>7</v>
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),13.0)</f>
+        <v>13</v>
       </c>
       <c r="D28" s="61">
         <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),12.0)</f>
         <v>12</v>
       </c>
       <c r="E28" s="61">
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),7.0)</f>
+        <v>7</v>
+      </c>
+      <c r="F28" s="61">
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),3.0)</f>
+        <v>3</v>
+      </c>
+      <c r="G28" s="61">
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0)</f>
+        <v>0</v>
+      </c>
+      <c r="H28" s="61">
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),38.0)</f>
+        <v>38</v>
+      </c>
+      <c r="I28" s="60" t="str">
+        <f t="shared" si="1"/>
+        <v>▮▮▮▮▮▮▮▯▯▯▯▯▯▯▯▯▯▯▯▯▯▯▯▯▯▯▯▯▯▯</v>
+      </c>
+      <c r="J28" s="62">
+        <f t="shared" si="2"/>
+        <v>12.7</v>
+      </c>
+      <c r="K28" s="62">
+        <f t="shared" si="3"/>
+        <v>79</v>
+      </c>
+      <c r="L28" s="60" t="s">
+        <v>70</v>
+      </c>
+      <c r="M28" s="60">
+        <f>SUMIF(Spelarstatistik!A$2:A179, L28, Spelarstatistik!B$2:B179)
+</f>
+        <v>0</v>
+      </c>
+      <c r="N28" s="60">
+        <f>SUMIF(Spelarstatistik!A$2:A179, L28, Spelarstatistik!C$2:C179)
+</f>
+        <v>0</v>
+      </c>
+      <c r="O28" s="60">
+        <f>SUMIF(Spelarstatistik!A$2:A179, L28, Spelarstatistik!D$2:D179)
+</f>
+        <v>4</v>
+      </c>
+      <c r="P28" s="60">
+        <f>SUMIF(Spelarstatistik!A$2:A179, L28, Spelarstatistik!E$2:E179)
+</f>
+        <v>14</v>
+      </c>
+      <c r="Q28" s="60">
+        <f>COUNTIF(Spelarstatistik!A$2:A179, L28)
+</f>
+        <v>3</v>
+      </c>
+      <c r="R28" s="60">
+        <f>SUMIF(Matcher!AC$5:AC179, L28, Matcher!AH$5:AH179)
+</f>
+        <v>0</v>
+      </c>
+      <c r="S28" s="60">
+        <f t="shared" si="4"/>
+        <v>17</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="60" t="str">
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"George T")</f>
+        <v>George T</v>
+      </c>
+      <c r="B29" s="64">
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),4.0)</f>
+        <v>4</v>
+      </c>
+      <c r="C29" s="64">
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),7.0)</f>
+        <v>7</v>
+      </c>
+      <c r="D29" s="61">
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),12.0)</f>
+        <v>12</v>
+      </c>
+      <c r="E29" s="61">
         <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),14.0)</f>
         <v>14</v>
       </c>
-      <c r="F28" s="61">
+      <c r="F29" s="61">
         <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),4.0)</f>
         <v>4</v>
       </c>
-      <c r="G28" s="61">
+      <c r="G29" s="61">
         <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0)</f>
         <v>0</v>
-      </c>
-      <c r="H28" s="61">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),37.0)</f>
-        <v>37</v>
-      </c>
-      <c r="I28" s="60" t="str">
-        <f t="shared" si="1"/>
-        <v>▮▮▮▮▮▮▯▯▯▯▯▯▯▯▯▯▯▯▯▯▯▯▯▯▯▯▯▯▯▯</v>
-      </c>
-      <c r="J28" s="62">
-        <f t="shared" si="2"/>
-        <v>9.3</v>
-      </c>
-      <c r="K28" s="62">
-        <f t="shared" si="3"/>
-        <v>64</v>
-      </c>
-      <c r="L28" s="60" t="s">
-        <v>36</v>
-      </c>
-      <c r="M28" s="60">
-        <f>SUMIF(Spelarstatistik!A$2:A179, L28, Spelarstatistik!B$2:B179)
-</f>
-        <v>36</v>
-      </c>
-      <c r="N28" s="60">
-        <f>SUMIF(Spelarstatistik!A$2:A179, L28, Spelarstatistik!C$2:C179)
-</f>
-        <v>37</v>
-      </c>
-      <c r="O28" s="60">
-        <f>SUMIF(Spelarstatistik!A$2:A179, L28, Spelarstatistik!D$2:D179)
-</f>
-        <v>52</v>
-      </c>
-      <c r="P28" s="60">
-        <f>SUMIF(Spelarstatistik!A$2:A179, L28, Spelarstatistik!E$2:E179)
-</f>
-        <v>32</v>
-      </c>
-      <c r="Q28" s="60">
-        <f>COUNTIF(Spelarstatistik!A$2:A179, L28)
-</f>
-        <v>15</v>
-      </c>
-      <c r="R28" s="60">
-        <f>SUMIF(Matcher!AC$5:AC179, L28, Matcher!AH$5:AH179)
-</f>
-        <v>0</v>
-      </c>
-      <c r="S28" s="60">
-        <f t="shared" si="4"/>
-        <v>174</v>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" s="60" t="str">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"Ture H")</f>
-        <v>Ture H</v>
-      </c>
-      <c r="B29" s="64">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),2.0)</f>
-        <v>2</v>
-      </c>
-      <c r="C29" s="64">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),1.0)</f>
-        <v>1</v>
-      </c>
-      <c r="D29" s="61">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),15.0)</f>
-        <v>15</v>
-      </c>
-      <c r="E29" s="61">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),8.0)</f>
-        <v>8</v>
-      </c>
-      <c r="F29" s="61">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),3.0)</f>
-        <v>3</v>
-      </c>
-      <c r="G29" s="61">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),23.0)</f>
-        <v>23</v>
       </c>
       <c r="H29" s="61">
         <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),37.0)</f>
@@ -33738,14 +33735,14 @@
       </c>
       <c r="J29" s="62">
         <f t="shared" si="2"/>
-        <v>12.3</v>
+        <v>9.3</v>
       </c>
       <c r="K29" s="62">
         <f t="shared" si="3"/>
-        <v>79</v>
+        <v>64</v>
       </c>
       <c r="L29" s="60" t="s">
-        <v>71</v>
+        <v>42</v>
       </c>
       <c r="M29" s="60">
         <f>SUMIF(Spelarstatistik!A$2:A179, L29, Spelarstatistik!B$2:B179)
@@ -33755,65 +33752,65 @@
       <c r="N29" s="60">
         <f>SUMIF(Spelarstatistik!A$2:A179, L29, Spelarstatistik!C$2:C179)
 </f>
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="O29" s="60">
         <f>SUMIF(Spelarstatistik!A$2:A179, L29, Spelarstatistik!D$2:D179)
 </f>
-        <v>4</v>
+        <v>21</v>
       </c>
       <c r="P29" s="60">
         <f>SUMIF(Spelarstatistik!A$2:A179, L29, Spelarstatistik!E$2:E179)
 </f>
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="Q29" s="60">
         <f>COUNTIF(Spelarstatistik!A$2:A179, L29)
 </f>
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="R29" s="60">
         <f>SUMIF(Matcher!AC$5:AC179, L29, Matcher!AH$5:AH179)
 </f>
-        <v>0</v>
+        <v>20</v>
       </c>
       <c r="S29" s="60">
         <f t="shared" si="4"/>
-        <v>17</v>
+        <v>63</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="60" t="str">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"Benjamin L")</f>
-        <v>Benjamin L</v>
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"Ture H")</f>
+        <v>Ture H</v>
       </c>
       <c r="B30" s="64">
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),2.0)</f>
+        <v>2</v>
+      </c>
+      <c r="C30" s="64">
         <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),1.0)</f>
         <v>1</v>
-      </c>
-      <c r="C30" s="64">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),2.0)</f>
-        <v>2</v>
       </c>
       <c r="D30" s="61">
         <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),15.0)</f>
         <v>15</v>
       </c>
       <c r="E30" s="61">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),11.0)</f>
-        <v>11</v>
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),8.0)</f>
+        <v>8</v>
       </c>
       <c r="F30" s="61">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),5.0)</f>
-        <v>5</v>
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),3.0)</f>
+        <v>3</v>
       </c>
       <c r="G30" s="61">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0)</f>
-        <v>0</v>
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),23.0)</f>
+        <v>23</v>
       </c>
       <c r="H30" s="61">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),36.0)</f>
-        <v>36</v>
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),37.0)</f>
+        <v>37</v>
       </c>
       <c r="I30" s="60" t="str">
         <f t="shared" si="1"/>
@@ -33821,48 +33818,48 @@
       </c>
       <c r="J30" s="62">
         <f t="shared" si="2"/>
-        <v>7.2</v>
+        <v>12.3</v>
       </c>
       <c r="K30" s="62">
         <f t="shared" si="3"/>
-        <v>51</v>
+        <v>79</v>
       </c>
       <c r="L30" s="60" t="s">
-        <v>42</v>
+        <v>72</v>
       </c>
       <c r="M30" s="60">
         <f>SUMIF(Spelarstatistik!A$2:A179, L30, Spelarstatistik!B$2:B179)
 </f>
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="N30" s="60">
         <f>SUMIF(Spelarstatistik!A$2:A179, L30, Spelarstatistik!C$2:C179)
 </f>
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="O30" s="60">
         <f>SUMIF(Spelarstatistik!A$2:A179, L30, Spelarstatistik!D$2:D179)
 </f>
-        <v>21</v>
+        <v>15</v>
       </c>
       <c r="P30" s="60">
         <f>SUMIF(Spelarstatistik!A$2:A179, L30, Spelarstatistik!E$2:E179)
 </f>
-        <v>15</v>
+        <v>7</v>
       </c>
       <c r="Q30" s="60">
         <f>COUNTIF(Spelarstatistik!A$2:A179, L30)
 </f>
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="R30" s="60">
         <f>SUMIF(Matcher!AC$5:AC179, L30, Matcher!AH$5:AH179)
 </f>
-        <v>20</v>
+        <v>0</v>
       </c>
       <c r="S30" s="60">
         <f t="shared" si="4"/>
-        <v>63</v>
+        <v>35</v>
       </c>
     </row>
     <row r="31">
@@ -33911,22 +33908,22 @@
         <v>79</v>
       </c>
       <c r="L31" s="60" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="M31" s="60">
         <f>SUMIF(Spelarstatistik!A$2:A179, L31, Spelarstatistik!B$2:B179)
 </f>
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="N31" s="60">
         <f>SUMIF(Spelarstatistik!A$2:A179, L31, Spelarstatistik!C$2:C179)
 </f>
-        <v>4</v>
+        <v>13</v>
       </c>
       <c r="O31" s="60">
         <f>SUMIF(Spelarstatistik!A$2:A179, L31, Spelarstatistik!D$2:D179)
 </f>
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="P31" s="60">
         <f>SUMIF(Spelarstatistik!A$2:A179, L31, Spelarstatistik!E$2:E179)
@@ -33945,7 +33942,7 @@
       </c>
       <c r="S31" s="60">
         <f t="shared" si="4"/>
-        <v>35</v>
+        <v>38</v>
       </c>
     </row>
     <row r="32">
@@ -33994,32 +33991,32 @@
         <v>77</v>
       </c>
       <c r="L32" s="60" t="s">
-        <v>67</v>
+        <v>75</v>
       </c>
       <c r="M32" s="60">
         <f>SUMIF(Spelarstatistik!A$2:A179, L32, Spelarstatistik!B$2:B179)
 </f>
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="N32" s="60">
         <f>SUMIF(Spelarstatistik!A$2:A179, L32, Spelarstatistik!C$2:C179)
 </f>
-        <v>13</v>
+        <v>0</v>
       </c>
       <c r="O32" s="60">
         <f>SUMIF(Spelarstatistik!A$2:A179, L32, Spelarstatistik!D$2:D179)
 </f>
-        <v>12</v>
+        <v>3</v>
       </c>
       <c r="P32" s="60">
         <f>SUMIF(Spelarstatistik!A$2:A179, L32, Spelarstatistik!E$2:E179)
 </f>
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="Q32" s="60">
         <f>COUNTIF(Spelarstatistik!A$2:A179, L32)
 </f>
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="R32" s="60">
         <f>SUMIF(Matcher!AC$5:AC179, L32, Matcher!AH$5:AH179)
@@ -34028,7 +34025,7 @@
       </c>
       <c r="S32" s="60">
         <f t="shared" si="4"/>
-        <v>38</v>
+        <v>7</v>
       </c>
     </row>
     <row r="33">
@@ -34077,12 +34074,12 @@
         <v>59</v>
       </c>
       <c r="L33" s="60" t="s">
-        <v>76</v>
+        <v>56</v>
       </c>
       <c r="M33" s="60">
         <f>SUMIF(Spelarstatistik!A$2:A179, L33, Spelarstatistik!B$2:B179)
 </f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N33" s="60">
         <f>SUMIF(Spelarstatistik!A$2:A179, L33, Spelarstatistik!C$2:C179)
@@ -34092,12 +34089,12 @@
       <c r="O33" s="60">
         <f>SUMIF(Spelarstatistik!A$2:A179, L33, Spelarstatistik!D$2:D179)
 </f>
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="P33" s="60">
         <f>SUMIF(Spelarstatistik!A$2:A179, L33, Spelarstatistik!E$2:E179)
 </f>
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="Q33" s="60">
         <f>COUNTIF(Spelarstatistik!A$2:A179, L33)
@@ -34160,32 +34157,32 @@
         <v>78</v>
       </c>
       <c r="L34" s="60" t="s">
-        <v>56</v>
+        <v>63</v>
       </c>
       <c r="M34" s="60">
         <f>SUMIF(Spelarstatistik!A$2:A179, L34, Spelarstatistik!B$2:B179)
 </f>
-        <v>1</v>
+        <v>9</v>
       </c>
       <c r="N34" s="60">
         <f>SUMIF(Spelarstatistik!A$2:A179, L34, Spelarstatistik!C$2:C179)
 </f>
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="O34" s="60">
         <f>SUMIF(Spelarstatistik!A$2:A179, L34, Spelarstatistik!D$2:D179)
 </f>
-        <v>1</v>
+        <v>9</v>
       </c>
       <c r="P34" s="60">
         <f>SUMIF(Spelarstatistik!A$2:A179, L34, Spelarstatistik!E$2:E179)
 </f>
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="Q34" s="60">
         <f>COUNTIF(Spelarstatistik!A$2:A179, L34)
 </f>
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="R34" s="60">
         <f>SUMIF(Matcher!AC$5:AC179, L34, Matcher!AH$5:AH179)
@@ -34194,7 +34191,7 @@
       </c>
       <c r="S34" s="60">
         <f t="shared" si="4"/>
-        <v>7</v>
+        <v>34</v>
       </c>
     </row>
     <row r="35">
@@ -34243,32 +34240,32 @@
         <v>60</v>
       </c>
       <c r="L35" s="60" t="s">
-        <v>63</v>
+        <v>73</v>
       </c>
       <c r="M35" s="60">
         <f>SUMIF(Spelarstatistik!A$2:A179, L35, Spelarstatistik!B$2:B179)
 </f>
-        <v>9</v>
+        <v>5</v>
       </c>
       <c r="N35" s="60">
         <f>SUMIF(Spelarstatistik!A$2:A179, L35, Spelarstatistik!C$2:C179)
 </f>
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="O35" s="60">
         <f>SUMIF(Spelarstatistik!A$2:A179, L35, Spelarstatistik!D$2:D179)
 </f>
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="P35" s="60">
         <f>SUMIF(Spelarstatistik!A$2:A179, L35, Spelarstatistik!E$2:E179)
 </f>
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="Q35" s="60">
         <f>COUNTIF(Spelarstatistik!A$2:A179, L35)
 </f>
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="R35" s="60">
         <f>SUMIF(Matcher!AC$5:AC179, L35, Matcher!AH$5:AH179)
@@ -34277,7 +34274,7 @@
       </c>
       <c r="S35" s="60">
         <f t="shared" si="4"/>
-        <v>34</v>
+        <v>16</v>
       </c>
     </row>
     <row r="36">
@@ -34326,22 +34323,22 @@
         <v>57</v>
       </c>
       <c r="L36" s="60" t="s">
-        <v>74</v>
+        <v>43</v>
       </c>
       <c r="M36" s="60">
         <f>SUMIF(Spelarstatistik!A$2:A179, L36, Spelarstatistik!B$2:B179)
 </f>
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="N36" s="60">
         <f>SUMIF(Spelarstatistik!A$2:A179, L36, Spelarstatistik!C$2:C179)
 </f>
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="O36" s="60">
         <f>SUMIF(Spelarstatistik!A$2:A179, L36, Spelarstatistik!D$2:D179)
 </f>
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="P36" s="60">
         <f>SUMIF(Spelarstatistik!A$2:A179, L36, Spelarstatistik!E$2:E179)
@@ -34360,7 +34357,7 @@
       </c>
       <c r="S36" s="60">
         <f t="shared" si="4"/>
-        <v>16</v>
+        <v>12</v>
       </c>
     </row>
     <row r="37">
@@ -34409,27 +34406,27 @@
         <v>39</v>
       </c>
       <c r="L37" s="60" t="s">
-        <v>43</v>
+        <v>54</v>
       </c>
       <c r="M37" s="60">
         <f>SUMIF(Spelarstatistik!A$2:A179, L37, Spelarstatistik!B$2:B179)
 </f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="N37" s="60">
         <f>SUMIF(Spelarstatistik!A$2:A179, L37, Spelarstatistik!C$2:C179)
 </f>
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="O37" s="60">
         <f>SUMIF(Spelarstatistik!A$2:A179, L37, Spelarstatistik!D$2:D179)
 </f>
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="P37" s="60">
         <f>SUMIF(Spelarstatistik!A$2:A179, L37, Spelarstatistik!E$2:E179)
 </f>
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="Q37" s="60">
         <f>COUNTIF(Spelarstatistik!A$2:A179, L37)
@@ -34443,7 +34440,7 @@
       </c>
       <c r="S37" s="60">
         <f t="shared" si="4"/>
-        <v>12</v>
+        <v>8</v>
       </c>
     </row>
     <row r="38">
@@ -34492,27 +34489,27 @@
         <v>77</v>
       </c>
       <c r="L38" s="60" t="s">
-        <v>54</v>
+        <v>74</v>
       </c>
       <c r="M38" s="60">
         <f>SUMIF(Spelarstatistik!A$2:A179, L38, Spelarstatistik!B$2:B179)
 </f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N38" s="60">
         <f>SUMIF(Spelarstatistik!A$2:A179, L38, Spelarstatistik!C$2:C179)
 </f>
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="O38" s="60">
         <f>SUMIF(Spelarstatistik!A$2:A179, L38, Spelarstatistik!D$2:D179)
 </f>
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="P38" s="60">
         <f>SUMIF(Spelarstatistik!A$2:A179, L38, Spelarstatistik!E$2:E179)
 </f>
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="Q38" s="60">
         <f>COUNTIF(Spelarstatistik!A$2:A179, L38)
@@ -34575,32 +34572,32 @@
         <v>77</v>
       </c>
       <c r="L39" s="60" t="s">
-        <v>75</v>
+        <v>32</v>
       </c>
       <c r="M39" s="60">
         <f>SUMIF(Spelarstatistik!A$2:A179, L39, Spelarstatistik!B$2:B179)
 </f>
-        <v>1</v>
+        <v>14</v>
       </c>
       <c r="N39" s="60">
         <f>SUMIF(Spelarstatistik!A$2:A179, L39, Spelarstatistik!C$2:C179)
 </f>
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="O39" s="60">
         <f>SUMIF(Spelarstatistik!A$2:A179, L39, Spelarstatistik!D$2:D179)
 </f>
-        <v>4</v>
+        <v>13</v>
       </c>
       <c r="P39" s="60">
         <f>SUMIF(Spelarstatistik!A$2:A179, L39, Spelarstatistik!E$2:E179)
 </f>
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="Q39" s="60">
         <f>COUNTIF(Spelarstatistik!A$2:A179, L39)
 </f>
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="R39" s="60">
         <f>SUMIF(Matcher!AC$5:AC179, L39, Matcher!AH$5:AH179)
@@ -34609,7 +34606,7 @@
       </c>
       <c r="S39" s="60">
         <f t="shared" si="4"/>
-        <v>8</v>
+        <v>45</v>
       </c>
     </row>
     <row r="40">
@@ -34658,32 +34655,32 @@
         <v>77</v>
       </c>
       <c r="L40" s="60" t="s">
-        <v>32</v>
+        <v>61</v>
       </c>
       <c r="M40" s="60">
         <f>SUMIF(Spelarstatistik!A$2:A179, L40, Spelarstatistik!B$2:B179)
 </f>
-        <v>14</v>
+        <v>0</v>
       </c>
       <c r="N40" s="60">
         <f>SUMIF(Spelarstatistik!A$2:A179, L40, Spelarstatistik!C$2:C179)
 </f>
-        <v>9</v>
+        <v>1</v>
       </c>
       <c r="O40" s="60">
         <f>SUMIF(Spelarstatistik!A$2:A179, L40, Spelarstatistik!D$2:D179)
 </f>
-        <v>13</v>
+        <v>1</v>
       </c>
       <c r="P40" s="60">
         <f>SUMIF(Spelarstatistik!A$2:A179, L40, Spelarstatistik!E$2:E179)
 </f>
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="Q40" s="60">
         <f>COUNTIF(Spelarstatistik!A$2:A179, L40)
 </f>
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="R40" s="60">
         <f>SUMIF(Matcher!AC$5:AC179, L40, Matcher!AH$5:AH179)
@@ -34692,7 +34689,7 @@
       </c>
       <c r="S40" s="60">
         <f t="shared" si="4"/>
-        <v>45</v>
+        <v>7</v>
       </c>
     </row>
     <row r="41">
@@ -34741,32 +34738,32 @@
         <v>76</v>
       </c>
       <c r="L41" s="60" t="s">
-        <v>61</v>
+        <v>35</v>
       </c>
       <c r="M41" s="60">
         <f>SUMIF(Spelarstatistik!A$2:A179, L41, Spelarstatistik!B$2:B179)
 </f>
-        <v>0</v>
+        <v>28</v>
       </c>
       <c r="N41" s="60">
         <f>SUMIF(Spelarstatistik!A$2:A179, L41, Spelarstatistik!C$2:C179)
 </f>
-        <v>1</v>
+        <v>22</v>
       </c>
       <c r="O41" s="60">
         <f>SUMIF(Spelarstatistik!A$2:A179, L41, Spelarstatistik!D$2:D179)
 </f>
-        <v>1</v>
+        <v>48</v>
       </c>
       <c r="P41" s="60">
         <f>SUMIF(Spelarstatistik!A$2:A179, L41, Spelarstatistik!E$2:E179)
 </f>
-        <v>4</v>
+        <v>50</v>
       </c>
       <c r="Q41" s="60">
         <f>COUNTIF(Spelarstatistik!A$2:A179, L41)
 </f>
-        <v>1</v>
+        <v>17</v>
       </c>
       <c r="R41" s="60">
         <f>SUMIF(Matcher!AC$5:AC179, L41, Matcher!AH$5:AH179)
@@ -34775,7 +34772,7 @@
       </c>
       <c r="S41" s="60">
         <f t="shared" si="4"/>
-        <v>7</v>
+        <v>159</v>
       </c>
     </row>
     <row r="42">
@@ -34824,32 +34821,32 @@
         <v>76</v>
       </c>
       <c r="L42" s="60" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="M42" s="60">
         <f>SUMIF(Spelarstatistik!A$2:A179, L42, Spelarstatistik!B$2:B179)
 </f>
-        <v>28</v>
+        <v>2</v>
       </c>
       <c r="N42" s="60">
         <f>SUMIF(Spelarstatistik!A$2:A179, L42, Spelarstatistik!C$2:C179)
 </f>
-        <v>22</v>
+        <v>2</v>
       </c>
       <c r="O42" s="60">
         <f>SUMIF(Spelarstatistik!A$2:A179, L42, Spelarstatistik!D$2:D179)
 </f>
-        <v>48</v>
+        <v>4</v>
       </c>
       <c r="P42" s="60">
         <f>SUMIF(Spelarstatistik!A$2:A179, L42, Spelarstatistik!E$2:E179)
 </f>
-        <v>50</v>
+        <v>5</v>
       </c>
       <c r="Q42" s="60">
         <f>COUNTIF(Spelarstatistik!A$2:A179, L42)
 </f>
-        <v>17</v>
+        <v>1</v>
       </c>
       <c r="R42" s="60">
         <f>SUMIF(Matcher!AC$5:AC179, L42, Matcher!AH$5:AH179)
@@ -34858,7 +34855,7 @@
       </c>
       <c r="S42" s="60">
         <f t="shared" si="4"/>
-        <v>159</v>
+        <v>11</v>
       </c>
     </row>
     <row r="43">
@@ -34907,32 +34904,32 @@
         <v>72</v>
       </c>
       <c r="L43" s="60" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
       <c r="M43" s="60">
         <f>SUMIF(Spelarstatistik!A$2:A179, L43, Spelarstatistik!B$2:B179)
 </f>
-        <v>2</v>
+        <v>16</v>
       </c>
       <c r="N43" s="60">
         <f>SUMIF(Spelarstatistik!A$2:A179, L43, Spelarstatistik!C$2:C179)
 </f>
-        <v>2</v>
+        <v>23</v>
       </c>
       <c r="O43" s="60">
         <f>SUMIF(Spelarstatistik!A$2:A179, L43, Spelarstatistik!D$2:D179)
 </f>
-        <v>4</v>
+        <v>48</v>
       </c>
       <c r="P43" s="60">
         <f>SUMIF(Spelarstatistik!A$2:A179, L43, Spelarstatistik!E$2:E179)
 </f>
-        <v>5</v>
+        <v>35</v>
       </c>
       <c r="Q43" s="60">
         <f>COUNTIF(Spelarstatistik!A$2:A179, L43)
 </f>
-        <v>1</v>
+        <v>14</v>
       </c>
       <c r="R43" s="60">
         <f>SUMIF(Matcher!AC$5:AC179, L43, Matcher!AH$5:AH179)
@@ -34941,7 +34938,7 @@
       </c>
       <c r="S43" s="60">
         <f t="shared" si="4"/>
-        <v>11</v>
+        <v>133</v>
       </c>
     </row>
     <row r="44">
@@ -34990,32 +34987,32 @@
         <v>66</v>
       </c>
       <c r="L44" s="60" t="s">
-        <v>34</v>
+        <v>71</v>
       </c>
       <c r="M44" s="60">
         <f>SUMIF(Spelarstatistik!A$2:A179, L44, Spelarstatistik!B$2:B179)
 </f>
-        <v>16</v>
+        <v>6</v>
       </c>
       <c r="N44" s="60">
         <f>SUMIF(Spelarstatistik!A$2:A179, L44, Spelarstatistik!C$2:C179)
 </f>
-        <v>23</v>
+        <v>3</v>
       </c>
       <c r="O44" s="60">
         <f>SUMIF(Spelarstatistik!A$2:A179, L44, Spelarstatistik!D$2:D179)
 </f>
-        <v>48</v>
+        <v>10</v>
       </c>
       <c r="P44" s="60">
         <f>SUMIF(Spelarstatistik!A$2:A179, L44, Spelarstatistik!E$2:E179)
 </f>
-        <v>35</v>
+        <v>15</v>
       </c>
       <c r="Q44" s="60">
         <f>COUNTIF(Spelarstatistik!A$2:A179, L44)
 </f>
-        <v>14</v>
+        <v>4</v>
       </c>
       <c r="R44" s="60">
         <f>SUMIF(Matcher!AC$5:AC179, L44, Matcher!AH$5:AH179)
@@ -35024,13 +35021,13 @@
       </c>
       <c r="S44" s="60">
         <f t="shared" si="4"/>
-        <v>133</v>
+        <v>34</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="60" t="str">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"Benji L")</f>
-        <v>Benji L</v>
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"Mattias R")</f>
+        <v>Mattias R</v>
       </c>
       <c r="B45" s="61">
         <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0)</f>
@@ -35045,8 +35042,8 @@
         <v>1</v>
       </c>
       <c r="E45" s="61">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),3.0)</f>
-        <v>3</v>
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),7.0)</f>
+        <v>7</v>
       </c>
       <c r="F45" s="61">
         <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),1.0)</f>
@@ -35073,27 +35070,27 @@
         <v>53</v>
       </c>
       <c r="L45" s="60" t="s">
-        <v>72</v>
+        <v>51</v>
       </c>
       <c r="M45" s="60">
         <f>SUMIF(Spelarstatistik!A$2:A179, L45, Spelarstatistik!B$2:B179)
 </f>
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="N45" s="60">
         <f>SUMIF(Spelarstatistik!A$2:A179, L45, Spelarstatistik!C$2:C179)
 </f>
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="O45" s="60">
         <f>SUMIF(Spelarstatistik!A$2:A179, L45, Spelarstatistik!D$2:D179)
 </f>
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="P45" s="60">
         <f>SUMIF(Spelarstatistik!A$2:A179, L45, Spelarstatistik!E$2:E179)
 </f>
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="Q45" s="60">
         <f>COUNTIF(Spelarstatistik!A$2:A179, L45)
@@ -35107,29 +35104,29 @@
       </c>
       <c r="S45" s="60">
         <f t="shared" si="4"/>
-        <v>34</v>
+        <v>42</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="60" t="str">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"Mattias R")</f>
-        <v>Mattias R</v>
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"Mattias X")</f>
+        <v>Mattias X</v>
       </c>
       <c r="B46" s="61">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0)</f>
-        <v>0</v>
-      </c>
-      <c r="C46" s="61">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),2.0)</f>
-        <v>2</v>
-      </c>
-      <c r="D46" s="61">
         <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),1.0)</f>
         <v>1</v>
       </c>
+      <c r="C46" s="61">
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0)</f>
+        <v>0</v>
+      </c>
+      <c r="D46" s="61">
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),4.0)</f>
+        <v>4</v>
+      </c>
       <c r="E46" s="61">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),7.0)</f>
-        <v>7</v>
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),3.0)</f>
+        <v>3</v>
       </c>
       <c r="F46" s="61">
         <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),1.0)</f>
@@ -35156,63 +35153,63 @@
         <v>53</v>
       </c>
       <c r="L46" s="60" t="s">
-        <v>51</v>
+        <v>40</v>
       </c>
       <c r="M46" s="60">
         <f>SUMIF(Spelarstatistik!A$2:A179, L46, Spelarstatistik!B$2:B179)
 </f>
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="N46" s="60">
         <f>SUMIF(Spelarstatistik!A$2:A179, L46, Spelarstatistik!C$2:C179)
 </f>
-        <v>8</v>
+        <v>21</v>
       </c>
       <c r="O46" s="60">
         <f>SUMIF(Spelarstatistik!A$2:A179, L46, Spelarstatistik!D$2:D179)
 </f>
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="P46" s="60">
         <f>SUMIF(Spelarstatistik!A$2:A179, L46, Spelarstatistik!E$2:E179)
 </f>
-        <v>12</v>
+        <v>1</v>
       </c>
       <c r="Q46" s="60">
         <f>COUNTIF(Spelarstatistik!A$2:A179, L46)
 </f>
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="R46" s="60">
         <f>SUMIF(Matcher!AC$5:AC179, L46, Matcher!AH$5:AH179)
 </f>
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="S46" s="60">
         <f t="shared" si="4"/>
-        <v>42</v>
+        <v>71</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="60" t="str">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"Mattias X")</f>
-        <v>Mattias X</v>
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"Hampus W")</f>
+        <v>Hampus W</v>
       </c>
       <c r="B47" s="61">
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0)</f>
+        <v>0</v>
+      </c>
+      <c r="C47" s="61">
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0)</f>
+        <v>0</v>
+      </c>
+      <c r="D47" s="61">
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),3.0)</f>
+        <v>3</v>
+      </c>
+      <c r="E47" s="61">
         <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),1.0)</f>
         <v>1</v>
-      </c>
-      <c r="C47" s="61">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0)</f>
-        <v>0</v>
-      </c>
-      <c r="D47" s="61">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),4.0)</f>
-        <v>4</v>
-      </c>
-      <c r="E47" s="61">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),3.0)</f>
-        <v>3</v>
       </c>
       <c r="F47" s="61">
         <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),1.0)</f>
@@ -35223,8 +35220,8 @@
         <v>0</v>
       </c>
       <c r="H47" s="61">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),8.0)</f>
-        <v>8</v>
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),7.0)</f>
+        <v>7</v>
       </c>
       <c r="I47" s="60" t="str">
         <f t="shared" si="1"/>
@@ -35232,70 +35229,70 @@
       </c>
       <c r="J47" s="62">
         <f t="shared" si="2"/>
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="K47" s="62">
         <f t="shared" si="3"/>
-        <v>53</v>
+        <v>46</v>
       </c>
       <c r="L47" s="60" t="s">
-        <v>40</v>
+        <v>24</v>
       </c>
       <c r="M47" s="60">
         <f>SUMIF(Spelarstatistik!A$2:A179, L47, Spelarstatistik!B$2:B179)
 </f>
-        <v>0</v>
+        <v>11</v>
       </c>
       <c r="N47" s="60">
         <f>SUMIF(Spelarstatistik!A$2:A179, L47, Spelarstatistik!C$2:C179)
 </f>
-        <v>21</v>
+        <v>29</v>
       </c>
       <c r="O47" s="60">
         <f>SUMIF(Spelarstatistik!A$2:A179, L47, Spelarstatistik!D$2:D179)
 </f>
-        <v>4</v>
+        <v>28</v>
       </c>
       <c r="P47" s="60">
         <f>SUMIF(Spelarstatistik!A$2:A179, L47, Spelarstatistik!E$2:E179)
 </f>
-        <v>1</v>
+        <v>40</v>
       </c>
       <c r="Q47" s="60">
         <f>COUNTIF(Spelarstatistik!A$2:A179, L47)
 </f>
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="R47" s="60">
         <f>SUMIF(Matcher!AC$5:AC179, L47, Matcher!AH$5:AH179)
 </f>
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="S47" s="60">
         <f t="shared" si="4"/>
-        <v>71</v>
+        <v>104</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="60" t="str">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"Hampus W")</f>
-        <v>Hampus W</v>
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"Immanuel A")</f>
+        <v>Immanuel A</v>
       </c>
       <c r="B48" s="61">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0)</f>
-        <v>0</v>
-      </c>
-      <c r="C48" s="61">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0)</f>
-        <v>0</v>
-      </c>
-      <c r="D48" s="61">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),3.0)</f>
-        <v>3</v>
-      </c>
-      <c r="E48" s="61">
         <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),1.0)</f>
         <v>1</v>
+      </c>
+      <c r="C48" s="61">
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),1.0)</f>
+        <v>1</v>
+      </c>
+      <c r="D48" s="61">
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0)</f>
+        <v>0</v>
+      </c>
+      <c r="E48" s="61">
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),7.0)</f>
+        <v>7</v>
       </c>
       <c r="F48" s="61">
         <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),1.0)</f>
@@ -35322,32 +35319,32 @@
         <v>46</v>
       </c>
       <c r="L48" s="60" t="s">
-        <v>24</v>
+        <v>52</v>
       </c>
       <c r="M48" s="60">
         <f>SUMIF(Spelarstatistik!A$2:A179, L48, Spelarstatistik!B$2:B179)
 </f>
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="N48" s="60">
         <f>SUMIF(Spelarstatistik!A$2:A179, L48, Spelarstatistik!C$2:C179)
 </f>
-        <v>29</v>
+        <v>8</v>
       </c>
       <c r="O48" s="60">
         <f>SUMIF(Spelarstatistik!A$2:A179, L48, Spelarstatistik!D$2:D179)
 </f>
-        <v>28</v>
+        <v>18</v>
       </c>
       <c r="P48" s="60">
         <f>SUMIF(Spelarstatistik!A$2:A179, L48, Spelarstatistik!E$2:E179)
 </f>
-        <v>40</v>
+        <v>21</v>
       </c>
       <c r="Q48" s="60">
         <f>COUNTIF(Spelarstatistik!A$2:A179, L48)
 </f>
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="R48" s="60">
         <f>SUMIF(Matcher!AC$5:AC179, L48, Matcher!AH$5:AH179)
@@ -35356,29 +35353,29 @@
       </c>
       <c r="S48" s="60">
         <f t="shared" si="4"/>
-        <v>104</v>
+        <v>62</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="60" t="str">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"Immanuel A")</f>
-        <v>Immanuel A</v>
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"Jonathan X")</f>
+        <v>Jonathan X</v>
       </c>
       <c r="B49" s="61">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),1.0)</f>
-        <v>1</v>
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0)</f>
+        <v>0</v>
       </c>
       <c r="C49" s="61">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),1.0)</f>
-        <v>1</v>
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0)</f>
+        <v>0</v>
       </c>
       <c r="D49" s="61">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0)</f>
-        <v>0</v>
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),3.0)</f>
+        <v>3</v>
       </c>
       <c r="E49" s="61">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),7.0)</f>
-        <v>7</v>
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),5.0)</f>
+        <v>5</v>
       </c>
       <c r="F49" s="61">
         <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),1.0)</f>
@@ -35405,7 +35402,7 @@
         <v>46</v>
       </c>
       <c r="L49" s="60" t="s">
-        <v>52</v>
+        <v>29</v>
       </c>
       <c r="M49" s="60">
         <f>SUMIF(Spelarstatistik!A$2:A179, L49, Spelarstatistik!B$2:B179)
@@ -35415,22 +35412,22 @@
       <c r="N49" s="60">
         <f>SUMIF(Spelarstatistik!A$2:A179, L49, Spelarstatistik!C$2:C179)
 </f>
-        <v>8</v>
+        <v>11</v>
       </c>
       <c r="O49" s="60">
         <f>SUMIF(Spelarstatistik!A$2:A179, L49, Spelarstatistik!D$2:D179)
 </f>
-        <v>18</v>
+        <v>34</v>
       </c>
       <c r="P49" s="60">
         <f>SUMIF(Spelarstatistik!A$2:A179, L49, Spelarstatistik!E$2:E179)
 </f>
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="Q49" s="60">
         <f>COUNTIF(Spelarstatistik!A$2:A179, L49)
 </f>
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="R49" s="60">
         <f>SUMIF(Matcher!AC$5:AC179, L49, Matcher!AH$5:AH179)
@@ -35439,29 +35436,29 @@
       </c>
       <c r="S49" s="60">
         <f t="shared" si="4"/>
-        <v>62</v>
+        <v>88</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="60" t="str">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"Jonathan X")</f>
-        <v>Jonathan X</v>
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"Karvan X")</f>
+        <v>Karvan X</v>
       </c>
       <c r="B50" s="61">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0)</f>
-        <v>0</v>
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),1.0)</f>
+        <v>1</v>
       </c>
       <c r="C50" s="61">
         <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0)</f>
         <v>0</v>
       </c>
       <c r="D50" s="61">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),3.0)</f>
-        <v>3</v>
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),1.0)</f>
+        <v>1</v>
       </c>
       <c r="E50" s="61">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),5.0)</f>
-        <v>5</v>
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),1.0)</f>
+        <v>1</v>
       </c>
       <c r="F50" s="61">
         <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),1.0)</f>
@@ -35488,32 +35485,32 @@
         <v>46</v>
       </c>
       <c r="L50" s="60" t="s">
-        <v>29</v>
+        <v>44</v>
       </c>
       <c r="M50" s="60">
         <f>SUMIF(Spelarstatistik!A$2:A179, L50, Spelarstatistik!B$2:B179)
 </f>
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="N50" s="60">
         <f>SUMIF(Spelarstatistik!A$2:A179, L50, Spelarstatistik!C$2:C179)
 </f>
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="O50" s="60">
         <f>SUMIF(Spelarstatistik!A$2:A179, L50, Spelarstatistik!D$2:D179)
 </f>
-        <v>34</v>
+        <v>15</v>
       </c>
       <c r="P50" s="60">
         <f>SUMIF(Spelarstatistik!A$2:A179, L50, Spelarstatistik!E$2:E179)
 </f>
-        <v>23</v>
+        <v>8</v>
       </c>
       <c r="Q50" s="60">
         <f>COUNTIF(Spelarstatistik!A$2:A179, L50)
 </f>
-        <v>10</v>
+        <v>4</v>
       </c>
       <c r="R50" s="60">
         <f>SUMIF(Matcher!AC$5:AC179, L50, Matcher!AH$5:AH179)
@@ -35522,29 +35519,29 @@
       </c>
       <c r="S50" s="60">
         <f t="shared" si="4"/>
-        <v>88</v>
+        <v>42</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="60" t="str">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"Karvan X")</f>
-        <v>Karvan X</v>
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"Moaaz T")</f>
+        <v>Moaaz T</v>
       </c>
       <c r="B51" s="61">
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0)</f>
+        <v>0</v>
+      </c>
+      <c r="C51" s="61">
         <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),1.0)</f>
         <v>1</v>
-      </c>
-      <c r="C51" s="61">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0)</f>
-        <v>0</v>
       </c>
       <c r="D51" s="61">
         <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),1.0)</f>
         <v>1</v>
       </c>
       <c r="E51" s="61">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),1.0)</f>
-        <v>1</v>
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),4.0)</f>
+        <v>4</v>
       </c>
       <c r="F51" s="61">
         <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),1.0)</f>
@@ -35571,17 +35568,17 @@
         <v>46</v>
       </c>
       <c r="L51" s="60" t="s">
-        <v>44</v>
+        <v>62</v>
       </c>
       <c r="M51" s="60">
         <f>SUMIF(Spelarstatistik!A$2:A179, L51, Spelarstatistik!B$2:B179)
 </f>
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="N51" s="60">
         <f>SUMIF(Spelarstatistik!A$2:A179, L51, Spelarstatistik!C$2:C179)
 </f>
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="O51" s="60">
         <f>SUMIF(Spelarstatistik!A$2:A179, L51, Spelarstatistik!D$2:D179)
@@ -35596,38 +35593,38 @@
       <c r="Q51" s="60">
         <f>COUNTIF(Spelarstatistik!A$2:A179, L51)
 </f>
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="R51" s="60">
         <f>SUMIF(Matcher!AC$5:AC179, L51, Matcher!AH$5:AH179)
 </f>
-        <v>0</v>
+        <v>23</v>
       </c>
       <c r="S51" s="60">
         <f t="shared" si="4"/>
-        <v>42</v>
+        <v>37</v>
       </c>
     </row>
     <row r="52">
       <c r="A52" s="60" t="str">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"Moaaz T")</f>
-        <v>Moaaz T</v>
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"Achillie X")</f>
+        <v>Achillie X</v>
       </c>
       <c r="B52" s="61">
         <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0)</f>
         <v>0</v>
       </c>
       <c r="C52" s="61">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),1.0)</f>
-        <v>1</v>
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0)</f>
+        <v>0</v>
       </c>
       <c r="D52" s="61">
         <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),1.0)</f>
         <v>1</v>
       </c>
       <c r="E52" s="61">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),4.0)</f>
-        <v>4</v>
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),3.0)</f>
+        <v>3</v>
       </c>
       <c r="F52" s="61">
         <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),1.0)</f>
@@ -35638,8 +35635,8 @@
         <v>0</v>
       </c>
       <c r="H52" s="61">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),7.0)</f>
-        <v>7</v>
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),6.0)</f>
+        <v>6</v>
       </c>
       <c r="I52" s="60" t="str">
         <f t="shared" si="1"/>
@@ -35647,54 +35644,54 @@
       </c>
       <c r="J52" s="62">
         <f t="shared" si="2"/>
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="K52" s="62">
         <f t="shared" si="3"/>
-        <v>46</v>
+        <v>40</v>
       </c>
       <c r="L52" s="60" t="s">
-        <v>62</v>
+        <v>50</v>
       </c>
       <c r="M52" s="60">
         <f>SUMIF(Spelarstatistik!A$2:A179, L52, Spelarstatistik!B$2:B179)
 </f>
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="N52" s="60">
         <f>SUMIF(Spelarstatistik!A$2:A179, L52, Spelarstatistik!C$2:C179)
 </f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="O52" s="60">
         <f>SUMIF(Spelarstatistik!A$2:A179, L52, Spelarstatistik!D$2:D179)
 </f>
-        <v>15</v>
+        <v>0</v>
       </c>
       <c r="P52" s="60">
         <f>SUMIF(Spelarstatistik!A$2:A179, L52, Spelarstatistik!E$2:E179)
 </f>
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="Q52" s="60">
         <f>COUNTIF(Spelarstatistik!A$2:A179, L52)
 </f>
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="R52" s="60">
         <f>SUMIF(Matcher!AC$5:AC179, L52, Matcher!AH$5:AH179)
 </f>
-        <v>23</v>
+        <v>0</v>
       </c>
       <c r="S52" s="60">
         <f t="shared" si="4"/>
-        <v>37</v>
+        <v>5</v>
       </c>
     </row>
     <row r="53">
       <c r="A53" s="60" t="str">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"Achillie X")</f>
-        <v>Achillie X</v>
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"William X")</f>
+        <v>William X</v>
       </c>
       <c r="B53" s="61">
         <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0)</f>
@@ -35705,12 +35702,12 @@
         <v>0</v>
       </c>
       <c r="D53" s="61">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),1.0)</f>
-        <v>1</v>
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0)</f>
+        <v>0</v>
       </c>
       <c r="E53" s="61">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),3.0)</f>
-        <v>3</v>
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),7.0)</f>
+        <v>7</v>
       </c>
       <c r="F53" s="61">
         <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),1.0)</f>
@@ -35721,8 +35718,8 @@
         <v>0</v>
       </c>
       <c r="H53" s="61">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),6.0)</f>
-        <v>6</v>
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),5.0)</f>
+        <v>5</v>
       </c>
       <c r="I53" s="60" t="str">
         <f t="shared" si="1"/>
@@ -35730,39 +35727,39 @@
       </c>
       <c r="J53" s="62">
         <f t="shared" si="2"/>
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="K53" s="62">
         <f t="shared" si="3"/>
-        <v>40</v>
+        <v>33</v>
       </c>
       <c r="L53" s="60" t="s">
-        <v>50</v>
+        <v>26</v>
       </c>
       <c r="M53" s="60">
         <f>SUMIF(Spelarstatistik!A$2:A179, L53, Spelarstatistik!B$2:B179)
 </f>
-        <v>0</v>
+        <v>16</v>
       </c>
       <c r="N53" s="60">
         <f>SUMIF(Spelarstatistik!A$2:A179, L53, Spelarstatistik!C$2:C179)
 </f>
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="O53" s="60">
         <f>SUMIF(Spelarstatistik!A$2:A179, L53, Spelarstatistik!D$2:D179)
 </f>
-        <v>0</v>
+        <v>13</v>
       </c>
       <c r="P53" s="60">
         <f>SUMIF(Spelarstatistik!A$2:A179, L53, Spelarstatistik!E$2:E179)
 </f>
-        <v>7</v>
+        <v>47</v>
       </c>
       <c r="Q53" s="60">
         <f>COUNTIF(Spelarstatistik!A$2:A179, L53)
 </f>
-        <v>1</v>
+        <v>12</v>
       </c>
       <c r="R53" s="60">
         <f>SUMIF(Matcher!AC$5:AC179, L53, Matcher!AH$5:AH179)
@@ -35771,90 +35768,64 @@
       </c>
       <c r="S53" s="60">
         <f t="shared" si="4"/>
-        <v>5</v>
+        <v>92</v>
       </c>
     </row>
     <row r="54">
-      <c r="A54" s="60" t="str">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"William X")</f>
-        <v>William X</v>
-      </c>
-      <c r="B54" s="61">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0)</f>
-        <v>0</v>
-      </c>
-      <c r="C54" s="61">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0)</f>
-        <v>0</v>
-      </c>
-      <c r="D54" s="61">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0)</f>
-        <v>0</v>
-      </c>
-      <c r="E54" s="61">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),7.0)</f>
-        <v>7</v>
-      </c>
-      <c r="F54" s="61">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),1.0)</f>
-        <v>1</v>
-      </c>
-      <c r="G54" s="61">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0)</f>
-        <v>0</v>
-      </c>
-      <c r="H54" s="61">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),5.0)</f>
-        <v>5</v>
-      </c>
+      <c r="A54" s="60"/>
+      <c r="B54" s="61"/>
+      <c r="C54" s="61"/>
+      <c r="D54" s="61"/>
+      <c r="E54" s="61"/>
+      <c r="F54" s="61"/>
+      <c r="G54" s="61"/>
+      <c r="H54" s="61"/>
       <c r="I54" s="60" t="str">
         <f t="shared" si="1"/>
-        <v>▮▯▯▯▯▯▯▯▯▯▯▯▯▯▯▯▯▯▯▯▯▯▯▯▯▯▯▯▯▯</v>
-      </c>
-      <c r="J54" s="62">
+        <v/>
+      </c>
+      <c r="J54" s="62" t="str">
         <f t="shared" si="2"/>
-        <v>5</v>
+        <v/>
       </c>
       <c r="K54" s="62">
         <f t="shared" si="3"/>
-        <v>33</v>
-      </c>
-      <c r="L54" s="60" t="s">
-        <v>26</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="L54" s="60"/>
       <c r="M54" s="60">
         <f>SUMIF(Spelarstatistik!A$2:A179, L54, Spelarstatistik!B$2:B179)
 </f>
-        <v>16</v>
+        <v>0</v>
       </c>
       <c r="N54" s="60">
         <f>SUMIF(Spelarstatistik!A$2:A179, L54, Spelarstatistik!C$2:C179)
 </f>
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="O54" s="60">
         <f>SUMIF(Spelarstatistik!A$2:A179, L54, Spelarstatistik!D$2:D179)
 </f>
-        <v>13</v>
+        <v>0</v>
       </c>
       <c r="P54" s="60">
         <f>SUMIF(Spelarstatistik!A$2:A179, L54, Spelarstatistik!E$2:E179)
 </f>
-        <v>47</v>
+        <v>0</v>
       </c>
       <c r="Q54" s="60">
         <f>COUNTIF(Spelarstatistik!A$2:A179, L54)
 </f>
-        <v>12</v>
+        <v>0</v>
       </c>
       <c r="R54" s="60">
         <f>SUMIF(Matcher!AC$5:AC179, L54, Matcher!AH$5:AH179)
 </f>
         <v>0</v>
       </c>
-      <c r="S54" s="60">
+      <c r="S54" s="60" t="str">
         <f t="shared" si="4"/>
-        <v>92</v>
+        <v/>
       </c>
     </row>
     <row r="55">
@@ -41908,19 +41879,19 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="58" t="s">
+        <v>81</v>
+      </c>
+      <c r="B1" s="58" t="s">
         <v>82</v>
       </c>
-      <c r="B1" s="58" t="s">
+      <c r="C1" s="59" t="s">
         <v>83</v>
       </c>
-      <c r="C1" s="59" t="s">
+      <c r="D1" s="59" t="s">
         <v>84</v>
       </c>
-      <c r="D1" s="59" t="s">
+      <c r="E1" s="59" t="s">
         <v>85</v>
-      </c>
-      <c r="E1" s="59" t="s">
-        <v>86</v>
       </c>
       <c r="F1" s="65" t="s">
         <v>2</v>
@@ -41929,7 +41900,7 @@
         <v>5</v>
       </c>
       <c r="H1" s="67" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="I1" s="68" t="s">
         <v>7</v>
@@ -41942,7 +41913,7 @@
         <v>5</v>
       </c>
       <c r="M1" s="67" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="N1" s="68" t="s">
         <v>7</v>
@@ -41950,18 +41921,18 @@
     </row>
     <row r="2">
       <c r="A2" s="70" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="C2" s="71"/>
       <c r="D2" s="71"/>
       <c r="E2" s="71"/>
       <c r="F2" s="24">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("IFERROR(ROUND(AVERAGE(FILTER('Poängligan'!$J$2:$J31, MATCH('Poängligan'!$A$2:$A31, F3:F31, 0))), 2), """")"),9.5)</f>
-        <v>9.5</v>
+        <f>IFERROR(__xludf.DUMMYFUNCTION("IFERROR(ROUND(AVERAGE(FILTER('Poängligan'!$J$2:$J31, MATCH('Poängligan'!$A$2:$A31, F3:F31, 0))), 2), """")"),11.43)</f>
+        <v>11.43</v>
       </c>
       <c r="G2" s="26">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("IFERROR(ROUND(AVERAGE(FILTER('Poängligan'!$J$2:$J31, MATCH('Poängligan'!$A$2:$A31, G3:G31, 0))), 2), """")"),10.9)</f>
-        <v>10.9</v>
+        <f>IFERROR(__xludf.DUMMYFUNCTION("IFERROR(ROUND(AVERAGE(FILTER('Poängligan'!$J$2:$J31, MATCH('Poängligan'!$A$2:$A31, G3:G31, 0))), 2), """")"),9.74)</f>
+        <v>9.74</v>
       </c>
       <c r="H2" s="28" t="str">
         <f>IFERROR(__xludf.DUMMYFUNCTION("IFERROR(ROUND(AVERAGE(FILTER('Poängligan'!$J$2:$J31, MATCH('Poängligan'!$A$2:$A31, H3:H31, 0))), 2), """")"),"")</f>
@@ -41998,12 +41969,12 @@
       </c>
       <c r="C3" s="75">
         <f>IF(ISBLANK(A3), "", RAND())</f>
-        <v>0.3148314606</v>
+        <v>0.5202665549</v>
       </c>
       <c r="D3" s="75">
         <f>IF(ISBLANK(A3), "", RANK(C3, $C$3:$C31))
 </f>
-        <v>14</v>
+        <v>8</v>
       </c>
       <c r="E3" s="75">
         <f>IF(ISBLANK(A3), "", MOD(D3-1, $B$3) + 1)
@@ -42012,13 +41983,13 @@
       </c>
       <c r="F3" s="38" t="str">
         <f>IFERROR(__xludf.DUMMYFUNCTION("SORT(IF($B$3&gt;=1, FILTER($A$3:$A31, $E$3:$E31=1), """"))
+"),"Daniel Ö")</f>
+        <v>Daniel Ö</v>
+      </c>
+      <c r="G3" s="35" t="str">
+        <f>IFERROR(__xludf.DUMMYFUNCTION("SORT(IF($B$3&gt;=2, FILTER($A$3:$A31, $E$3:$E31=2), """"))
 "),"Daniel K")</f>
         <v>Daniel K</v>
-      </c>
-      <c r="G3" s="35" t="str">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("SORT(IF($B$3&gt;=2, FILTER($A$3:$A31, $E$3:$E31=2), """"))
-"),"Daniel Ö")</f>
-        <v>Daniel Ö</v>
       </c>
       <c r="H3" s="76" t="str">
         <f>IFERROR(__xludf.DUMMYFUNCTION("SORT(IF($B$3&gt;=3, FILTER($A$3:$A31, $E$3:$E31=3), """"))
@@ -42028,7 +41999,7 @@
       <c r="I3" s="77"/>
       <c r="J3" s="78">
         <f>MAX(F2:I2)-MIN(F2:I2)</f>
-        <v>1.4</v>
+        <v>1.69</v>
       </c>
       <c r="K3" s="23" t="s">
         <v>24</v>
@@ -42037,7 +42008,7 @@
         <v>55</v>
       </c>
       <c r="M3" s="79" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="N3" s="80"/>
     </row>
@@ -42048,21 +42019,21 @@
       <c r="B4" s="81"/>
       <c r="C4" s="75">
         <f>IF(ISBLANK(#REF!), "", RAND())</f>
-        <v>0.4680562398</v>
+        <v>0.5263996699</v>
       </c>
       <c r="D4" s="75">
         <f>IF(ISBLANK(#REF!), "", RANK(C4, $C$3:$C31))
 </f>
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="E4" s="75">
         <f>IF(ISBLANK(#REF!), "", MOD(D4-1, $B$3) + 1)
 </f>
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F4" s="38" t="str">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"Emil A")</f>
-        <v>Emil A</v>
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"Isak L")</f>
+        <v>Isak L</v>
       </c>
       <c r="G4" s="35" t="str">
         <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"Dennis F")</f>
@@ -42072,7 +42043,7 @@
       <c r="I4" s="77"/>
       <c r="J4" s="78"/>
       <c r="K4" s="23" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="L4" s="25" t="s">
         <v>33</v>
@@ -42088,34 +42059,34 @@
       </c>
       <c r="C5" s="75">
         <f>IF(ISBLANK(A5), "", RAND())</f>
-        <v>0.9366905028</v>
+        <v>0.2170365783</v>
       </c>
       <c r="D5" s="75">
         <f>IF(ISBLANK(A5), "", RANK(C5, $C$3:$C31))
 </f>
-        <v>2</v>
+        <v>11</v>
       </c>
       <c r="E5" s="75">
         <f>IF(ISBLANK(A5), "", MOD(D5-1, $B$3) + 1)
 </f>
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F5" s="38" t="str">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"Ivan N")</f>
-        <v>Ivan N</v>
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"Jakob S")</f>
+        <v>Jakob S</v>
       </c>
       <c r="G5" s="35" t="str">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"Isak L")</f>
-        <v>Isak L</v>
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"Emil A")</f>
+        <v>Emil A</v>
       </c>
       <c r="H5" s="76"/>
       <c r="I5" s="77"/>
       <c r="J5" s="78"/>
       <c r="K5" s="23" t="s">
+        <v>90</v>
+      </c>
+      <c r="L5" s="25" t="s">
         <v>91</v>
-      </c>
-      <c r="L5" s="25" t="s">
-        <v>92</v>
       </c>
       <c r="M5" s="79" t="s">
         <v>34</v>
@@ -42128,32 +42099,32 @@
       </c>
       <c r="C6" s="75">
         <f t="shared" ref="C6:C10" si="1">IF(ISBLANK(#REF!), "", RAND())</f>
-        <v>0.6891027961</v>
+        <v>0.8037007033</v>
       </c>
       <c r="D6" s="75">
         <f t="shared" ref="D6:D10" si="2">IF(ISBLANK(#REF!), "", RANK(C6, $C$3:$C31))
 </f>
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="E6" s="75">
         <f t="shared" ref="E6:E10" si="3">IF(ISBLANK(#REF!), "", MOD(D6-1, $B$3) + 1)
 </f>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F6" s="38"/>
       <c r="G6" s="35" t="str">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"Jakob S")</f>
-        <v>Jakob S</v>
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"Ivan N")</f>
+        <v>Ivan N</v>
       </c>
       <c r="H6" s="76"/>
       <c r="I6" s="77"/>
       <c r="J6" s="78"/>
       <c r="K6" s="23"/>
       <c r="L6" s="25" t="s">
+        <v>92</v>
+      </c>
+      <c r="M6" s="79" t="s">
         <v>93</v>
-      </c>
-      <c r="M6" s="79" t="s">
-        <v>94</v>
       </c>
       <c r="N6" s="80"/>
     </row>
@@ -42163,15 +42134,15 @@
       </c>
       <c r="C7" s="75">
         <f t="shared" si="1"/>
-        <v>0.09131931008</v>
+        <v>0.3387795809</v>
       </c>
       <c r="D7" s="75">
         <f t="shared" si="2"/>
-        <v>16</v>
+        <v>9</v>
       </c>
       <c r="E7" s="75">
         <f t="shared" si="3"/>
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F7" s="38"/>
       <c r="G7" s="35" t="str">
@@ -42188,15 +42159,15 @@
     </row>
     <row r="8">
       <c r="A8" s="83" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="C8" s="75">
         <f t="shared" si="1"/>
-        <v>0.8698003284</v>
+        <v>0.3137351548</v>
       </c>
       <c r="D8" s="75">
         <f t="shared" si="2"/>
-        <v>4</v>
+        <v>10</v>
       </c>
       <c r="E8" s="75">
         <f t="shared" si="3"/>
@@ -42221,15 +42192,15 @@
       </c>
       <c r="C9" s="75">
         <f t="shared" si="1"/>
-        <v>0.379144493</v>
+        <v>0.2083219025</v>
       </c>
       <c r="D9" s="75">
         <f t="shared" si="2"/>
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="E9" s="75">
         <f t="shared" si="3"/>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F9" s="38"/>
       <c r="G9" s="35" t="str">
@@ -42250,11 +42221,11 @@
       </c>
       <c r="C10" s="75">
         <f t="shared" si="1"/>
-        <v>0.7413427507</v>
+        <v>0.7232311731</v>
       </c>
       <c r="D10" s="75">
         <f t="shared" si="2"/>
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="E10" s="75">
         <f t="shared" si="3"/>
@@ -42272,16 +42243,16 @@
     </row>
     <row r="11">
       <c r="A11" s="83" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="C11" s="75">
         <f>IF(ISBLANK(A4), "", RAND())</f>
-        <v>0.3819154476</v>
+        <v>0.08696658247</v>
       </c>
       <c r="D11" s="75">
         <f>IF(ISBLANK(A4), "", RANK(C11, $C$3:$C31))
 </f>
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="E11" s="75">
         <f>IF(ISBLANK(A4), "", MOD(D11-1, $B$3) + 1)
@@ -42304,17 +42275,17 @@
       </c>
       <c r="C12" s="75">
         <f t="shared" ref="C12:C16" si="4">IF(ISBLANK(#REF!), "", RAND())</f>
-        <v>0.4281421119</v>
+        <v>0.0227563889</v>
       </c>
       <c r="D12" s="75">
         <f t="shared" ref="D12:D16" si="5">IF(ISBLANK(#REF!), "", RANK(C12, $C$3:$C31))
 </f>
-        <v>11</v>
+        <v>16</v>
       </c>
       <c r="E12" s="75">
         <f t="shared" ref="E12:E16" si="6">IF(ISBLANK(#REF!), "", MOD(D12-1, $B$3) + 1)
 </f>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F12" s="38"/>
       <c r="G12" s="35"/>
@@ -42329,11 +42300,11 @@
     <row r="13">
       <c r="C13" s="75">
         <f t="shared" si="4"/>
-        <v>0.919163146</v>
+        <v>0.9802371123</v>
       </c>
       <c r="D13" s="75">
         <f t="shared" si="5"/>
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="E13" s="75">
         <f t="shared" si="6"/>
@@ -42352,11 +42323,11 @@
     <row r="14">
       <c r="C14" s="75">
         <f t="shared" si="4"/>
-        <v>0.6270726227</v>
+        <v>0.7775014491</v>
       </c>
       <c r="D14" s="75">
         <f t="shared" si="5"/>
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="E14" s="75">
         <f t="shared" si="6"/>
@@ -42376,11 +42347,11 @@
       <c r="A15" s="83"/>
       <c r="C15" s="75">
         <f t="shared" si="4"/>
-        <v>0.9971158409</v>
+        <v>0.0292258779</v>
       </c>
       <c r="D15" s="75">
         <f t="shared" si="5"/>
-        <v>1</v>
+        <v>15</v>
       </c>
       <c r="E15" s="75">
         <f t="shared" si="6"/>
@@ -42400,15 +42371,15 @@
       <c r="A16" s="73"/>
       <c r="C16" s="75">
         <f t="shared" si="4"/>
-        <v>0.1534634025</v>
+        <v>0.6076575476</v>
       </c>
       <c r="D16" s="75">
         <f t="shared" si="5"/>
-        <v>15</v>
+        <v>6</v>
       </c>
       <c r="E16" s="75">
         <f t="shared" si="6"/>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F16" s="38"/>
       <c r="G16" s="35"/>
@@ -42449,12 +42420,12 @@
     <row r="18">
       <c r="C18" s="75">
         <f>IF(ISBLANK(A10), "", RAND())</f>
-        <v>0.8618238355</v>
+        <v>0.1127683348</v>
       </c>
       <c r="D18" s="75">
         <f>IF(ISBLANK(A10), "", RANK(C18, $C$3:$C31))
 </f>
-        <v>5</v>
+        <v>13</v>
       </c>
       <c r="E18" s="75">
         <f>IF(ISBLANK(A10), "", MOD(D18-1, $B$3) + 1)
@@ -42474,17 +42445,17 @@
     <row r="19">
       <c r="C19" s="75">
         <f>IF(ISBLANK(A7), "", RAND())</f>
-        <v>0.6728814419</v>
+        <v>0.6136604293</v>
       </c>
       <c r="D19" s="75">
         <f>IF(ISBLANK(A7), "", RANK(C19, $C$3:$C31))
 </f>
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="E19" s="75">
         <f>IF(ISBLANK(A7), "", MOD(D19-1, $B$3) + 1)
 </f>
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F19" s="38"/>
       <c r="G19" s="35"/>
@@ -42993,7 +42964,7 @@
     </row>
     <row r="5">
       <c r="A5" s="20" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="B5" s="8">
         <v>3.0</v>
@@ -43007,7 +42978,7 @@
         <v>1.0</v>
       </c>
       <c r="E5" s="21" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="F5" s="22" t="str">
         <f t="shared" ref="F5:F23" si="2">IF(AND(B5 &lt;&gt; "", D5 &lt;&gt; ""), IF(B5 &gt; D5, A5, IF(D5 &gt; B5, E5, "Oavgjort")), "")</f>
@@ -43102,7 +43073,7 @@
     </row>
     <row r="6">
       <c r="A6" s="20" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="B6" s="8">
         <v>2.0</v>
@@ -43115,7 +43086,7 @@
         <v>0.0</v>
       </c>
       <c r="E6" s="21" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="F6" s="22" t="str">
         <f t="shared" si="2"/>
@@ -43191,7 +43162,7 @@
     </row>
     <row r="7">
       <c r="A7" s="20" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="B7" s="8">
         <v>3.0</v>
@@ -43204,7 +43175,7 @@
         <v>1.0</v>
       </c>
       <c r="E7" s="21" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="F7" s="22" t="str">
         <f t="shared" si="2"/>
@@ -43270,7 +43241,7 @@
     </row>
     <row r="8">
       <c r="A8" s="20" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="B8" s="8">
         <v>5.0</v>
@@ -43282,7 +43253,7 @@
         <v>2.0</v>
       </c>
       <c r="E8" s="21" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="F8" s="22" t="str">
         <f t="shared" si="2"/>
@@ -43494,7 +43465,7 @@
         <v/>
       </c>
       <c r="H11" s="23" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="I11" s="9">
         <v>2.0</v>
@@ -43628,7 +43599,7 @@
         <v/>
       </c>
       <c r="H13" s="23" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="I13" s="9">
         <v>0.0</v>
@@ -44419,7 +44390,7 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="58" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="B1" s="58" t="s">
         <v>3</v>
@@ -47553,8 +47524,8 @@
     </row>
     <row r="143">
       <c r="A143" s="81" t="str">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"Benji L")</f>
-        <v>Benji L</v>
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"Benjamin L")</f>
+        <v>Benjamin L</v>
       </c>
       <c r="B143" s="81">
         <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0)</f>
@@ -55511,19 +55482,19 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="58" t="s">
+        <v>81</v>
+      </c>
+      <c r="B1" s="58" t="s">
         <v>82</v>
       </c>
-      <c r="B1" s="58" t="s">
+      <c r="C1" s="59" t="s">
         <v>83</v>
       </c>
-      <c r="C1" s="59" t="s">
+      <c r="D1" s="59" t="s">
         <v>84</v>
       </c>
-      <c r="D1" s="59" t="s">
+      <c r="E1" s="59" t="s">
         <v>85</v>
-      </c>
-      <c r="E1" s="59" t="s">
-        <v>86</v>
       </c>
       <c r="F1" s="65" t="s">
         <v>2</v>
@@ -55532,10 +55503,10 @@
         <v>5</v>
       </c>
       <c r="H1" s="67" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="I1" s="69" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
     </row>
     <row r="2">
@@ -55547,27 +55518,27 @@
       </c>
       <c r="C2" s="75">
         <f t="shared" ref="C2:C30" si="1">IF(ISBLANK(A2), "", RAND())</f>
-        <v>0.9784831049</v>
+        <v>0.2136697829</v>
       </c>
       <c r="D2" s="75">
         <f t="shared" ref="D2:D30" si="2">IF(ISBLANK(A2), "", RANK(C2, $C$2:$C30))
 </f>
-        <v>1</v>
+        <v>14</v>
       </c>
       <c r="E2" s="75">
         <f t="shared" ref="E2:E30" si="3">IF(ISBLANK(A2), "", MOD(D2-1, $B$2) + 1)
 </f>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F2" s="38" t="str">
         <f>IFERROR(__xludf.DUMMYFUNCTION("SORT(IF($B$2&gt;=1, FILTER($A$2:$A30, $E$2:$E30=1), """"))
+"),"Benjamin L")</f>
+        <v>Benjamin L</v>
+      </c>
+      <c r="G2" s="35" t="str">
+        <f>IFERROR(__xludf.DUMMYFUNCTION("SORT(IF($B$2&gt;=2, FILTER($A$2:$A30, $E$2:$E30=2), """"))
 "),"Ali K")</f>
         <v>Ali K</v>
-      </c>
-      <c r="G2" s="35" t="str">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("SORT(IF($B$2&gt;=2, FILTER($A$2:$A30, $E$2:$E30=2), """"))
-"),"Benjamin L")</f>
-        <v>Benjamin L</v>
       </c>
       <c r="H2" s="76" t="str">
         <f>IFERROR(__xludf.DUMMYFUNCTION("SORT(IF($B$2&gt;=3, FILTER($A$2:$A30, $E$2:$E30=3), """"))
@@ -55582,28 +55553,28 @@
     </row>
     <row r="3">
       <c r="A3" s="74" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="B3" s="81"/>
       <c r="C3" s="75">
         <f t="shared" si="1"/>
-        <v>0.3231286287</v>
+        <v>0.1704035879</v>
       </c>
       <c r="D3" s="75">
         <f t="shared" si="2"/>
-        <v>13</v>
+        <v>16</v>
       </c>
       <c r="E3" s="75">
         <f t="shared" si="3"/>
         <v>1</v>
       </c>
       <c r="F3" s="38" t="str">
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"Erik N")</f>
+        <v>Erik N</v>
+      </c>
+      <c r="G3" s="35" t="str">
         <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"Aria A")</f>
         <v>Aria A</v>
-      </c>
-      <c r="G3" s="35" t="str">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"Daniel K")</f>
-        <v>Daniel K</v>
       </c>
       <c r="H3" s="76" t="str">
         <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"Ilir A")</f>
@@ -55617,57 +55588,57 @@
       </c>
       <c r="C4" s="75">
         <f t="shared" si="1"/>
-        <v>0.9168166841</v>
+        <v>0.9947260104</v>
       </c>
       <c r="D4" s="75">
         <f t="shared" si="2"/>
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="E4" s="75">
         <f t="shared" si="3"/>
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="F4" s="38" t="str">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"Erik N")</f>
-        <v>Erik N</v>
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"Hawsang")</f>
+        <v>Hawsang</v>
       </c>
       <c r="G4" s="35" t="str">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"Leo K")</f>
-        <v>Leo K</v>
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"Daniel K")</f>
+        <v>Daniel K</v>
       </c>
       <c r="H4" s="76" t="str">
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"Jakob S")</f>
+        <v>Jakob S</v>
+      </c>
+      <c r="I4" s="84"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="74" t="s">
+        <v>102</v>
+      </c>
+      <c r="C5" s="75">
+        <f t="shared" si="1"/>
+        <v>0.5227468208</v>
+      </c>
+      <c r="D5" s="75">
+        <f t="shared" si="2"/>
+        <v>7</v>
+      </c>
+      <c r="E5" s="75">
+        <f t="shared" si="3"/>
+        <v>1</v>
+      </c>
+      <c r="F5" s="38" t="str">
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"Oliver G")</f>
+        <v>Oliver G</v>
+      </c>
+      <c r="G5" s="35" t="str">
         <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"Isak H")</f>
         <v>Isak H</v>
       </c>
-      <c r="I4" s="84"/>
-    </row>
-    <row r="5">
-      <c r="A5" s="74" t="s">
-        <v>103</v>
-      </c>
-      <c r="C5" s="75">
-        <f t="shared" si="1"/>
-        <v>0.3793761972</v>
-      </c>
-      <c r="D5" s="75">
-        <f t="shared" si="2"/>
-        <v>11</v>
-      </c>
-      <c r="E5" s="75">
-        <f t="shared" si="3"/>
-        <v>2</v>
-      </c>
-      <c r="F5" s="38" t="str">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"Hawsang")</f>
-        <v>Hawsang</v>
-      </c>
-      <c r="G5" s="35" t="str">
+      <c r="H5" s="76" t="str">
         <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"Mattias R")</f>
         <v>Mattias R</v>
-      </c>
-      <c r="H5" s="76" t="str">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"Jakob S")</f>
-        <v>Jakob S</v>
       </c>
       <c r="I5" s="84"/>
     </row>
@@ -55677,53 +55648,53 @@
       </c>
       <c r="C6" s="75">
         <f t="shared" si="1"/>
-        <v>0.2676427643</v>
+        <v>0.5331402889</v>
       </c>
       <c r="D6" s="75">
         <f t="shared" si="2"/>
-        <v>15</v>
+        <v>6</v>
       </c>
       <c r="E6" s="75">
         <f t="shared" si="3"/>
         <v>3</v>
       </c>
       <c r="F6" s="38" t="str">
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"Oskar W ")</f>
+        <v>Oskar W </v>
+      </c>
+      <c r="G6" s="35" t="str">
         <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"Isak K")</f>
         <v>Isak K</v>
       </c>
-      <c r="G6" s="35" t="str">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"Oskar W ")</f>
-        <v>Oskar W </v>
-      </c>
       <c r="H6" s="76" t="str">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"Oliver G")</f>
-        <v>Oliver G</v>
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"Noor A")</f>
+        <v>Noor A</v>
       </c>
       <c r="I6" s="84"/>
     </row>
     <row r="7">
       <c r="A7" s="74" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="C7" s="75">
         <f t="shared" si="1"/>
-        <v>0.8199842739</v>
+        <v>0.4161944334</v>
       </c>
       <c r="D7" s="75">
         <f t="shared" si="2"/>
-        <v>6</v>
+        <v>12</v>
       </c>
       <c r="E7" s="75">
         <f t="shared" si="3"/>
         <v>3</v>
       </c>
       <c r="F7" s="38" t="str">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"Noor A")</f>
-        <v>Noor A</v>
-      </c>
-      <c r="G7" s="35" t="str">
         <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"Samuel P")</f>
         <v>Samuel P</v>
+      </c>
+      <c r="G7" s="35" t="str">
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"Leo K")</f>
+        <v>Leo K</v>
       </c>
       <c r="H7" s="76" t="str">
         <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"Oskar W")</f>
@@ -55737,15 +55708,15 @@
       </c>
       <c r="C8" s="75">
         <f t="shared" si="1"/>
-        <v>0.8410215323</v>
+        <v>0.7600807737</v>
       </c>
       <c r="D8" s="75">
         <f t="shared" si="2"/>
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="E8" s="75">
         <f t="shared" si="3"/>
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F8" s="38"/>
       <c r="G8" s="35"/>
@@ -55754,15 +55725,15 @@
     </row>
     <row r="9">
       <c r="A9" s="74" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="C9" s="75">
         <f t="shared" si="1"/>
-        <v>0.451282199</v>
+        <v>0.1786036519</v>
       </c>
       <c r="D9" s="75">
         <f t="shared" si="2"/>
-        <v>9</v>
+        <v>15</v>
       </c>
       <c r="E9" s="75">
         <f t="shared" si="3"/>
@@ -55775,19 +55746,19 @@
     </row>
     <row r="10">
       <c r="A10" s="74" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="C10" s="75">
         <f t="shared" si="1"/>
-        <v>0.4234036899</v>
+        <v>0.5895552492</v>
       </c>
       <c r="D10" s="75">
         <f t="shared" si="2"/>
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="E10" s="75">
         <f t="shared" si="3"/>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F10" s="38"/>
       <c r="G10" s="35"/>
@@ -55796,15 +55767,15 @@
     </row>
     <row r="11">
       <c r="A11" s="74" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="C11" s="75">
         <f t="shared" si="1"/>
-        <v>0.9706268946</v>
+        <v>0.4176573924</v>
       </c>
       <c r="D11" s="75">
         <f t="shared" si="2"/>
-        <v>2</v>
+        <v>11</v>
       </c>
       <c r="E11" s="75">
         <f t="shared" si="3"/>
@@ -55817,19 +55788,19 @@
     </row>
     <row r="12">
       <c r="A12" s="74" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="C12" s="75">
         <f t="shared" si="1"/>
-        <v>0.1720283767</v>
+        <v>0.8772373488</v>
       </c>
       <c r="D12" s="75">
         <f t="shared" si="2"/>
-        <v>16</v>
+        <v>2</v>
       </c>
       <c r="E12" s="75">
         <f t="shared" si="3"/>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F12" s="38"/>
       <c r="G12" s="35"/>
@@ -55842,15 +55813,15 @@
       </c>
       <c r="C13" s="75">
         <f t="shared" si="1"/>
-        <v>0.5350232918</v>
+        <v>0.3920584981</v>
       </c>
       <c r="D13" s="75">
         <f t="shared" si="2"/>
-        <v>8</v>
+        <v>13</v>
       </c>
       <c r="E13" s="75">
         <f t="shared" si="3"/>
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F13" s="38"/>
       <c r="G13" s="35"/>
@@ -55863,11 +55834,11 @@
       </c>
       <c r="C14" s="75">
         <f t="shared" si="1"/>
-        <v>0.2830013859</v>
+        <v>0.1124892657</v>
       </c>
       <c r="D14" s="75">
         <f t="shared" si="2"/>
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="E14" s="75">
         <f t="shared" si="3"/>
@@ -55884,15 +55855,15 @@
       </c>
       <c r="C15" s="75">
         <f t="shared" si="1"/>
-        <v>0.1564530896</v>
+        <v>0.4458137299</v>
       </c>
       <c r="D15" s="75">
         <f t="shared" si="2"/>
-        <v>17</v>
+        <v>10</v>
       </c>
       <c r="E15" s="75">
         <f t="shared" si="3"/>
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F15" s="38"/>
       <c r="G15" s="35"/>
@@ -55905,7 +55876,7 @@
       </c>
       <c r="C16" s="75">
         <f t="shared" si="1"/>
-        <v>0.05630396419</v>
+        <v>0.08766517966</v>
       </c>
       <c r="D16" s="75">
         <f t="shared" si="2"/>
@@ -55922,19 +55893,19 @@
     </row>
     <row r="17">
       <c r="A17" s="74" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="C17" s="75">
         <f t="shared" si="1"/>
-        <v>0.8858178894</v>
+        <v>0.4885155945</v>
       </c>
       <c r="D17" s="75">
         <f t="shared" si="2"/>
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="E17" s="75">
         <f t="shared" si="3"/>
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="F17" s="38"/>
       <c r="G17" s="35"/>
@@ -55943,19 +55914,19 @@
     </row>
     <row r="18">
       <c r="A18" s="74" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="C18" s="75">
         <f t="shared" si="1"/>
-        <v>0.3364702658</v>
+        <v>0.4958134977</v>
       </c>
       <c r="D18" s="75">
         <f t="shared" si="2"/>
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="E18" s="75">
         <f t="shared" si="3"/>
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F18" s="38"/>
       <c r="G18" s="35"/>
@@ -55964,15 +55935,15 @@
     </row>
     <row r="19">
       <c r="A19" s="74" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="C19" s="75">
         <f t="shared" si="1"/>
-        <v>0.6224517186</v>
+        <v>0.7529781488</v>
       </c>
       <c r="D19" s="75">
         <f t="shared" si="2"/>
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="E19" s="75">
         <f t="shared" si="3"/>

</xml_diff>